<commit_message>
update OPPM plan, unified SRS
</commit_message>
<xml_diff>
--- a/Task 2/OPPM_Plan.xlsx
+++ b/Task 2/OPPM_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kohaku\Downloads\LAB301\Task 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02B79D8F-C000-4A78-99AE-328D79A7A00D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC7DB633-2284-4261-BC2E-03E1593735D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -334,7 +334,7 @@
     <numFmt numFmtId="167" formatCode="_([$€-2]* #,##0.00_);_([$€-2]* \(#,##0.00\);_([$€-2]* &quot;-&quot;??_)"/>
     <numFmt numFmtId="168" formatCode="_(&quot;$&quot;* #"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -497,12 +497,6 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -2034,6 +2028,131 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="65" xfId="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="43" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="69" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="70" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="71" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="63" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="49" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="4" fillId="0" borderId="55" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="4" fillId="0" borderId="48" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="4" fillId="0" borderId="72" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="4" fillId="0" borderId="73" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="49" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="50" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2073,11 +2192,31 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="17" fontId="4" fillId="0" borderId="55" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="55" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="55" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="48" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="67" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="66" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="4" fillId="8" borderId="55" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="17" fontId="4" fillId="0" borderId="48" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="17" fontId="4" fillId="8" borderId="48" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -2101,153 +2240,8 @@
       <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="49" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="63" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="49" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="50" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="65" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="68" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="4" fillId="0" borderId="72" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="4" fillId="0" borderId="73" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="55" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="67" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="55" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="48" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="66" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="43" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="4" fillId="8" borderId="55" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="4" fillId="8" borderId="48" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="69" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="70" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="71" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -2414,20 +2408,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="mediumGray">
-          <fgColor indexed="10"/>
-          <bgColor indexed="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="mediumGray">
           <fgColor indexed="42"/>
@@ -2439,6 +2419,20 @@
       <fill>
         <patternFill patternType="mediumGray">
           <fgColor indexed="43"/>
+          <bgColor indexed="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="mediumGray">
+          <fgColor indexed="10"/>
           <bgColor indexed="9"/>
         </patternFill>
       </fill>
@@ -2918,7 +2912,7 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:noFill/>
             </a14:hiddenFill>
           </a:ext>
@@ -2972,7 +2966,7 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:noFill/>
             </a14:hiddenFill>
           </a:ext>
@@ -3328,14 +3322,14 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="3175">
+            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="3175">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -3394,7 +3388,7 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:noFill/>
             </a14:hiddenFill>
           </a:ext>
@@ -3448,7 +3442,7 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:noFill/>
             </a14:hiddenFill>
           </a:ext>
@@ -3502,7 +3496,7 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:noFill/>
             </a14:hiddenFill>
           </a:ext>
@@ -4069,27 +4063,27 @@
     <row r="3" spans="2:27" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="14"/>
       <c r="D3" s="15"/>
-      <c r="E3" s="161" t="s">
+      <c r="E3" s="193" t="s">
         <v>31</v>
       </c>
-      <c r="F3" s="162"/>
-      <c r="G3" s="162"/>
-      <c r="H3" s="162"/>
-      <c r="I3" s="162"/>
-      <c r="J3" s="162"/>
-      <c r="K3" s="162"/>
-      <c r="L3" s="162"/>
-      <c r="M3" s="162"/>
-      <c r="N3" s="162"/>
-      <c r="O3" s="162"/>
-      <c r="P3" s="162"/>
-      <c r="Q3" s="162"/>
-      <c r="R3" s="162"/>
-      <c r="S3" s="162"/>
-      <c r="T3" s="162"/>
-      <c r="U3" s="162"/>
-      <c r="V3" s="162"/>
-      <c r="W3" s="163"/>
+      <c r="F3" s="194"/>
+      <c r="G3" s="194"/>
+      <c r="H3" s="194"/>
+      <c r="I3" s="194"/>
+      <c r="J3" s="194"/>
+      <c r="K3" s="194"/>
+      <c r="L3" s="194"/>
+      <c r="M3" s="194"/>
+      <c r="N3" s="194"/>
+      <c r="O3" s="194"/>
+      <c r="P3" s="194"/>
+      <c r="Q3" s="194"/>
+      <c r="R3" s="194"/>
+      <c r="S3" s="194"/>
+      <c r="T3" s="194"/>
+      <c r="U3" s="194"/>
+      <c r="V3" s="194"/>
+      <c r="W3" s="195"/>
       <c r="Y3" s="12"/>
       <c r="Z3" s="13"/>
       <c r="AA3" s="13"/>
@@ -4098,60 +4092,60 @@
       <c r="B4" s="17"/>
       <c r="C4" s="18"/>
       <c r="D4" s="18"/>
-      <c r="E4" s="164"/>
-      <c r="F4" s="165"/>
-      <c r="G4" s="165"/>
-      <c r="H4" s="165"/>
-      <c r="I4" s="165"/>
-      <c r="J4" s="165"/>
-      <c r="K4" s="165"/>
-      <c r="L4" s="165"/>
-      <c r="M4" s="165"/>
-      <c r="N4" s="165"/>
-      <c r="O4" s="165"/>
-      <c r="P4" s="165"/>
-      <c r="Q4" s="165"/>
-      <c r="R4" s="165"/>
-      <c r="S4" s="165"/>
-      <c r="T4" s="165"/>
-      <c r="U4" s="165"/>
-      <c r="V4" s="165"/>
-      <c r="W4" s="166"/>
+      <c r="E4" s="196"/>
+      <c r="F4" s="197"/>
+      <c r="G4" s="197"/>
+      <c r="H4" s="197"/>
+      <c r="I4" s="197"/>
+      <c r="J4" s="197"/>
+      <c r="K4" s="197"/>
+      <c r="L4" s="197"/>
+      <c r="M4" s="197"/>
+      <c r="N4" s="197"/>
+      <c r="O4" s="197"/>
+      <c r="P4" s="197"/>
+      <c r="Q4" s="197"/>
+      <c r="R4" s="197"/>
+      <c r="S4" s="197"/>
+      <c r="T4" s="197"/>
+      <c r="U4" s="197"/>
+      <c r="V4" s="197"/>
+      <c r="W4" s="198"/>
       <c r="Y4" s="19"/>
       <c r="Z4" s="20"/>
       <c r="AA4" s="20"/>
     </row>
     <row r="5" spans="2:27" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="167" t="s">
+      <c r="B5" s="199" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="168"/>
-      <c r="D5" s="169"/>
+      <c r="C5" s="200"/>
+      <c r="D5" s="201"/>
       <c r="E5" s="21"/>
       <c r="F5" s="22" t="s">
         <v>1</v>
       </c>
       <c r="G5" s="23"/>
       <c r="H5" s="23"/>
-      <c r="I5" s="170" t="s">
+      <c r="I5" s="202" t="s">
         <v>2</v>
       </c>
-      <c r="J5" s="171"/>
-      <c r="K5" s="171"/>
-      <c r="L5" s="171"/>
-      <c r="M5" s="171"/>
-      <c r="N5" s="171"/>
-      <c r="O5" s="171"/>
-      <c r="P5" s="171"/>
-      <c r="Q5" s="171"/>
-      <c r="R5" s="172"/>
-      <c r="S5" s="170" t="s">
+      <c r="J5" s="203"/>
+      <c r="K5" s="203"/>
+      <c r="L5" s="203"/>
+      <c r="M5" s="203"/>
+      <c r="N5" s="203"/>
+      <c r="O5" s="203"/>
+      <c r="P5" s="203"/>
+      <c r="Q5" s="203"/>
+      <c r="R5" s="204"/>
+      <c r="S5" s="202" t="s">
         <v>3</v>
       </c>
-      <c r="T5" s="171"/>
-      <c r="U5" s="171"/>
-      <c r="V5" s="172"/>
-      <c r="W5" s="173"/>
+      <c r="T5" s="203"/>
+      <c r="U5" s="203"/>
+      <c r="V5" s="204"/>
+      <c r="W5" s="205"/>
     </row>
     <row r="6" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="25"/>
@@ -4162,11 +4156,11 @@
       <c r="E6" s="114">
         <v>1</v>
       </c>
-      <c r="F6" s="197" t="s">
+      <c r="F6" s="218" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="185"/>
-      <c r="H6" s="186"/>
+      <c r="G6" s="191"/>
+      <c r="H6" s="192"/>
       <c r="I6" s="112" t="s">
         <v>10</v>
       </c>
@@ -4179,7 +4173,7 @@
       <c r="P6" s="27"/>
       <c r="Q6" s="27"/>
       <c r="R6" s="27"/>
-      <c r="S6" s="206" t="s">
+      <c r="S6" s="163" t="s">
         <v>15</v>
       </c>
       <c r="T6" s="126"/>
@@ -4199,14 +4193,14 @@
       <c r="E7" s="125">
         <v>2</v>
       </c>
-      <c r="F7" s="198" t="s">
+      <c r="F7" s="171" t="s">
         <v>34</v>
       </c>
-      <c r="G7" s="187"/>
-      <c r="H7" s="188"/>
+      <c r="G7" s="172"/>
+      <c r="H7" s="173"/>
       <c r="I7" s="137"/>
       <c r="J7" s="112" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K7" s="37"/>
       <c r="L7" s="37"/>
@@ -4231,19 +4225,19 @@
       <c r="B8" s="25"/>
       <c r="C8" s="30"/>
       <c r="D8" s="112" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E8" s="115">
         <v>3</v>
       </c>
-      <c r="F8" s="198" t="s">
+      <c r="F8" s="171" t="s">
         <v>35</v>
       </c>
-      <c r="G8" s="187"/>
-      <c r="H8" s="188"/>
+      <c r="G8" s="172"/>
+      <c r="H8" s="173"/>
       <c r="I8" s="32"/>
       <c r="J8" s="112" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K8" s="33"/>
       <c r="L8" s="37"/>
@@ -4253,7 +4247,7 @@
       <c r="P8" s="33"/>
       <c r="Q8" s="33"/>
       <c r="R8" s="33"/>
-      <c r="S8" s="207" t="s">
+      <c r="S8" s="164" t="s">
         <v>15</v>
       </c>
       <c r="U8" s="116"/>
@@ -4272,11 +4266,11 @@
       <c r="E9" s="115">
         <v>4</v>
       </c>
-      <c r="F9" s="198" t="s">
+      <c r="F9" s="171" t="s">
         <v>36</v>
       </c>
-      <c r="G9" s="187"/>
-      <c r="H9" s="188"/>
+      <c r="G9" s="172"/>
+      <c r="H9" s="173"/>
       <c r="I9" s="32"/>
       <c r="J9" s="33"/>
       <c r="K9" s="112" t="s">
@@ -4309,11 +4303,11 @@
       <c r="E10" s="115">
         <v>5</v>
       </c>
-      <c r="F10" s="198" t="s">
+      <c r="F10" s="171" t="s">
         <v>37</v>
       </c>
-      <c r="G10" s="187"/>
-      <c r="H10" s="188"/>
+      <c r="G10" s="172"/>
+      <c r="H10" s="173"/>
       <c r="I10" s="32"/>
       <c r="J10" s="33"/>
       <c r="K10" s="35"/>
@@ -4326,7 +4320,7 @@
       <c r="P10" s="33"/>
       <c r="Q10" s="33"/>
       <c r="R10" s="33"/>
-      <c r="S10" s="207" t="s">
+      <c r="S10" s="164" t="s">
         <v>15</v>
       </c>
       <c r="T10" s="116"/>
@@ -4345,11 +4339,11 @@
       <c r="E11" s="115">
         <v>6</v>
       </c>
-      <c r="F11" s="198" t="s">
+      <c r="F11" s="171" t="s">
         <v>38</v>
       </c>
-      <c r="G11" s="187"/>
-      <c r="H11" s="188"/>
+      <c r="G11" s="172"/>
+      <c r="H11" s="173"/>
       <c r="I11" s="32"/>
       <c r="J11" s="33"/>
       <c r="K11" s="37"/>
@@ -4382,11 +4376,11 @@
       <c r="E12" s="115">
         <v>7</v>
       </c>
-      <c r="F12" s="198" t="s">
+      <c r="F12" s="171" t="s">
         <v>39</v>
       </c>
-      <c r="G12" s="187"/>
-      <c r="H12" s="188"/>
+      <c r="G12" s="172"/>
+      <c r="H12" s="173"/>
       <c r="I12" s="32"/>
       <c r="J12" s="33"/>
       <c r="K12" s="33"/>
@@ -4419,11 +4413,11 @@
       <c r="E13" s="115">
         <v>8</v>
       </c>
-      <c r="F13" s="198" t="s">
+      <c r="F13" s="171" t="s">
         <v>40</v>
       </c>
-      <c r="G13" s="187"/>
-      <c r="H13" s="188"/>
+      <c r="G13" s="172"/>
+      <c r="H13" s="173"/>
       <c r="I13" s="32"/>
       <c r="J13" s="33"/>
       <c r="K13" s="33"/>
@@ -4456,11 +4450,11 @@
       <c r="E14" s="115">
         <v>9</v>
       </c>
-      <c r="F14" s="198" t="s">
+      <c r="F14" s="171" t="s">
         <v>41</v>
       </c>
-      <c r="G14" s="187"/>
-      <c r="H14" s="188"/>
+      <c r="G14" s="172"/>
+      <c r="H14" s="173"/>
       <c r="I14" s="32"/>
       <c r="J14" s="33"/>
       <c r="K14" s="33"/>
@@ -4493,11 +4487,11 @@
       <c r="E15" s="115">
         <v>10</v>
       </c>
-      <c r="F15" s="198" t="s">
+      <c r="F15" s="171" t="s">
         <v>42</v>
       </c>
-      <c r="G15" s="187"/>
-      <c r="H15" s="188"/>
+      <c r="G15" s="172"/>
+      <c r="H15" s="173"/>
       <c r="I15" s="32"/>
       <c r="J15" s="33"/>
       <c r="K15" s="33"/>
@@ -4528,9 +4522,9 @@
       <c r="E16" s="115">
         <v>11</v>
       </c>
-      <c r="F16" s="198"/>
-      <c r="G16" s="187"/>
-      <c r="H16" s="188"/>
+      <c r="F16" s="171"/>
+      <c r="G16" s="172"/>
+      <c r="H16" s="173"/>
       <c r="I16" s="32"/>
       <c r="J16" s="33"/>
       <c r="K16" s="33"/>
@@ -4557,9 +4551,9 @@
       <c r="E17" s="115">
         <v>12</v>
       </c>
-      <c r="F17" s="198"/>
-      <c r="G17" s="187"/>
-      <c r="H17" s="188"/>
+      <c r="F17" s="171"/>
+      <c r="G17" s="172"/>
+      <c r="H17" s="173"/>
       <c r="I17" s="32"/>
       <c r="J17" s="33"/>
       <c r="K17" s="33"/>
@@ -4586,9 +4580,9 @@
       <c r="E18" s="115">
         <v>13</v>
       </c>
-      <c r="F18" s="198"/>
-      <c r="G18" s="187"/>
-      <c r="H18" s="188"/>
+      <c r="F18" s="171"/>
+      <c r="G18" s="172"/>
+      <c r="H18" s="173"/>
       <c r="I18" s="32"/>
       <c r="J18" s="33"/>
       <c r="K18" s="33"/>
@@ -4614,9 +4608,9 @@
       <c r="E19" s="115">
         <v>14</v>
       </c>
-      <c r="F19" s="198"/>
-      <c r="G19" s="187"/>
-      <c r="H19" s="188"/>
+      <c r="F19" s="171"/>
+      <c r="G19" s="172"/>
+      <c r="H19" s="173"/>
       <c r="I19" s="32"/>
       <c r="J19" s="33"/>
       <c r="K19" s="33"/>
@@ -4643,9 +4637,9 @@
       <c r="E20" s="115">
         <v>15</v>
       </c>
-      <c r="F20" s="198"/>
-      <c r="G20" s="187"/>
-      <c r="H20" s="188"/>
+      <c r="F20" s="171"/>
+      <c r="G20" s="172"/>
+      <c r="H20" s="173"/>
       <c r="I20" s="32"/>
       <c r="J20" s="33"/>
       <c r="K20" s="33"/>
@@ -4672,9 +4666,9 @@
       <c r="E21" s="115">
         <v>16</v>
       </c>
-      <c r="F21" s="198"/>
-      <c r="G21" s="187"/>
-      <c r="H21" s="188"/>
+      <c r="F21" s="171"/>
+      <c r="G21" s="172"/>
+      <c r="H21" s="173"/>
       <c r="I21" s="32"/>
       <c r="J21" s="33"/>
       <c r="K21" s="33"/>
@@ -4701,9 +4695,9 @@
       <c r="E22" s="115">
         <v>17</v>
       </c>
-      <c r="F22" s="198"/>
-      <c r="G22" s="187"/>
-      <c r="H22" s="188"/>
+      <c r="F22" s="171"/>
+      <c r="G22" s="172"/>
+      <c r="H22" s="173"/>
       <c r="I22" s="32"/>
       <c r="J22" s="33"/>
       <c r="K22" s="33"/>
@@ -4730,9 +4724,9 @@
       <c r="E23" s="115">
         <v>18</v>
       </c>
-      <c r="F23" s="198"/>
-      <c r="G23" s="187"/>
-      <c r="H23" s="188"/>
+      <c r="F23" s="171"/>
+      <c r="G23" s="172"/>
+      <c r="H23" s="173"/>
       <c r="I23" s="32"/>
       <c r="J23" s="33"/>
       <c r="K23" s="33"/>
@@ -4759,9 +4753,9 @@
       <c r="E24" s="115">
         <v>19</v>
       </c>
-      <c r="F24" s="198"/>
-      <c r="G24" s="187"/>
-      <c r="H24" s="188"/>
+      <c r="F24" s="171"/>
+      <c r="G24" s="172"/>
+      <c r="H24" s="173"/>
       <c r="I24" s="32"/>
       <c r="J24" s="33"/>
       <c r="K24" s="33"/>
@@ -4787,9 +4781,9 @@
       <c r="E25" s="115">
         <v>20</v>
       </c>
-      <c r="F25" s="198"/>
-      <c r="G25" s="187"/>
-      <c r="H25" s="188"/>
+      <c r="F25" s="171"/>
+      <c r="G25" s="172"/>
+      <c r="H25" s="173"/>
       <c r="I25" s="32"/>
       <c r="J25" s="33"/>
       <c r="K25" s="33"/>
@@ -4816,9 +4810,9 @@
       <c r="E26" s="115">
         <v>21</v>
       </c>
-      <c r="F26" s="198"/>
-      <c r="G26" s="187"/>
-      <c r="H26" s="188"/>
+      <c r="F26" s="171"/>
+      <c r="G26" s="172"/>
+      <c r="H26" s="173"/>
       <c r="I26" s="32"/>
       <c r="J26" s="33"/>
       <c r="K26" s="33"/>
@@ -4844,9 +4838,9 @@
       <c r="E27" s="115">
         <v>22</v>
       </c>
-      <c r="F27" s="198"/>
-      <c r="G27" s="187"/>
-      <c r="H27" s="188"/>
+      <c r="F27" s="171"/>
+      <c r="G27" s="172"/>
+      <c r="H27" s="173"/>
       <c r="I27" s="32"/>
       <c r="J27" s="33"/>
       <c r="K27" s="33"/>
@@ -4873,9 +4867,9 @@
       <c r="E28" s="115">
         <v>23</v>
       </c>
-      <c r="F28" s="198"/>
-      <c r="G28" s="187"/>
-      <c r="H28" s="188"/>
+      <c r="F28" s="171"/>
+      <c r="G28" s="172"/>
+      <c r="H28" s="173"/>
       <c r="I28" s="32"/>
       <c r="J28" s="33"/>
       <c r="K28" s="33"/>
@@ -4900,9 +4894,9 @@
       <c r="E29" s="140">
         <v>24</v>
       </c>
-      <c r="F29" s="198"/>
-      <c r="G29" s="187"/>
-      <c r="H29" s="188"/>
+      <c r="F29" s="171"/>
+      <c r="G29" s="172"/>
+      <c r="H29" s="173"/>
       <c r="I29" s="141"/>
       <c r="J29" s="34"/>
       <c r="K29" s="34"/>
@@ -4928,9 +4922,9 @@
       <c r="E30" s="140">
         <v>25</v>
       </c>
-      <c r="F30" s="198"/>
-      <c r="G30" s="187"/>
-      <c r="H30" s="188"/>
+      <c r="F30" s="171"/>
+      <c r="G30" s="172"/>
+      <c r="H30" s="173"/>
       <c r="I30" s="141"/>
       <c r="J30" s="34"/>
       <c r="K30" s="34"/>
@@ -4955,9 +4949,9 @@
       <c r="C31" s="40"/>
       <c r="D31" s="41"/>
       <c r="E31" s="140"/>
-      <c r="F31" s="195"/>
-      <c r="G31" s="196"/>
-      <c r="H31" s="196"/>
+      <c r="F31" s="161"/>
+      <c r="G31" s="162"/>
+      <c r="H31" s="162"/>
       <c r="I31" s="141"/>
       <c r="J31" s="34"/>
       <c r="K31" s="34"/>
@@ -5015,11 +5009,11 @@
       <c r="E33" s="125">
         <v>1</v>
       </c>
-      <c r="F33" s="210" t="s">
+      <c r="F33" s="174" t="s">
         <v>54</v>
       </c>
-      <c r="G33" s="211"/>
-      <c r="H33" s="212"/>
+      <c r="G33" s="175"/>
+      <c r="H33" s="176"/>
       <c r="I33" s="56"/>
       <c r="J33" s="57"/>
       <c r="K33" s="57"/>
@@ -5046,11 +5040,11 @@
       <c r="E34" s="125">
         <v>2</v>
       </c>
-      <c r="F34" s="213" t="s">
+      <c r="F34" s="165" t="s">
         <v>53</v>
       </c>
-      <c r="G34" s="214"/>
-      <c r="H34" s="215"/>
+      <c r="G34" s="166"/>
+      <c r="H34" s="167"/>
       <c r="I34" s="56"/>
       <c r="J34" s="57"/>
       <c r="K34" s="57"/>
@@ -5077,11 +5071,11 @@
       <c r="E35" s="115">
         <v>3</v>
       </c>
-      <c r="F35" s="216" t="s">
+      <c r="F35" s="168" t="s">
         <v>55</v>
       </c>
-      <c r="G35" s="217"/>
-      <c r="H35" s="218"/>
+      <c r="G35" s="169"/>
+      <c r="H35" s="170"/>
       <c r="I35" s="58"/>
       <c r="J35" s="59"/>
       <c r="K35" s="59"/>
@@ -5108,9 +5102,9 @@
       <c r="E36" s="115">
         <v>4</v>
       </c>
-      <c r="F36" s="213"/>
-      <c r="G36" s="214"/>
-      <c r="H36" s="215"/>
+      <c r="F36" s="165"/>
+      <c r="G36" s="166"/>
+      <c r="H36" s="167"/>
       <c r="I36" s="58"/>
       <c r="J36" s="59"/>
       <c r="K36" s="59"/>
@@ -5137,9 +5131,9 @@
       <c r="E37" s="115">
         <v>5</v>
       </c>
-      <c r="F37" s="213"/>
-      <c r="G37" s="214"/>
-      <c r="H37" s="215"/>
+      <c r="F37" s="165"/>
+      <c r="G37" s="166"/>
+      <c r="H37" s="167"/>
       <c r="I37" s="58"/>
       <c r="J37" s="59"/>
       <c r="K37" s="59"/>
@@ -5244,188 +5238,188 @@
       <c r="AA40" s="29"/>
     </row>
     <row r="41" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B41" s="201" t="s">
+      <c r="B41" s="206" t="s">
         <v>32</v>
       </c>
-      <c r="C41" s="201" t="s">
+      <c r="C41" s="206" t="s">
         <v>57</v>
       </c>
-      <c r="D41" s="202" t="s">
+      <c r="D41" s="209" t="s">
         <v>56</v>
       </c>
       <c r="F41" s="87"/>
       <c r="G41" s="88"/>
       <c r="H41" s="88"/>
-      <c r="I41" s="208" t="s">
+      <c r="I41" s="211" t="s">
         <v>43</v>
       </c>
-      <c r="J41" s="174" t="s">
+      <c r="J41" s="182" t="s">
         <v>44</v>
       </c>
-      <c r="K41" s="174" t="s">
+      <c r="K41" s="182" t="s">
         <v>45</v>
       </c>
-      <c r="L41" s="174" t="s">
+      <c r="L41" s="182" t="s">
         <v>46</v>
       </c>
-      <c r="M41" s="174" t="s">
+      <c r="M41" s="182" t="s">
         <v>47</v>
       </c>
-      <c r="N41" s="199" t="s">
+      <c r="N41" s="184" t="s">
         <v>48</v>
       </c>
-      <c r="O41" s="199" t="s">
+      <c r="O41" s="184" t="s">
         <v>49</v>
       </c>
-      <c r="P41" s="199" t="s">
+      <c r="P41" s="184" t="s">
         <v>50</v>
       </c>
-      <c r="Q41" s="199" t="s">
+      <c r="Q41" s="184" t="s">
         <v>51</v>
       </c>
-      <c r="R41" s="199"/>
-      <c r="S41" s="178" t="s">
+      <c r="R41" s="184"/>
+      <c r="S41" s="215" t="s">
         <v>52</v>
       </c>
-      <c r="T41" s="181"/>
-      <c r="U41" s="181"/>
-      <c r="V41" s="181"/>
-      <c r="W41" s="192"/>
+      <c r="T41" s="179"/>
+      <c r="U41" s="179"/>
+      <c r="V41" s="179"/>
+      <c r="W41" s="187"/>
       <c r="Y41" s="28"/>
       <c r="Z41" s="29"/>
       <c r="AA41" s="29"/>
     </row>
     <row r="42" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="203"/>
-      <c r="C42" s="203"/>
-      <c r="D42" s="202"/>
+      <c r="B42" s="207"/>
+      <c r="C42" s="207"/>
+      <c r="D42" s="209"/>
       <c r="F42" s="89"/>
       <c r="G42" s="88"/>
       <c r="H42" s="88"/>
-      <c r="I42" s="208"/>
-      <c r="J42" s="174"/>
-      <c r="K42" s="174"/>
-      <c r="L42" s="174"/>
-      <c r="M42" s="174"/>
-      <c r="N42" s="199"/>
-      <c r="O42" s="199"/>
-      <c r="P42" s="199"/>
-      <c r="Q42" s="199"/>
-      <c r="R42" s="199"/>
-      <c r="S42" s="179"/>
-      <c r="T42" s="182"/>
-      <c r="U42" s="182"/>
-      <c r="V42" s="181"/>
-      <c r="W42" s="193"/>
+      <c r="I42" s="211"/>
+      <c r="J42" s="182"/>
+      <c r="K42" s="182"/>
+      <c r="L42" s="182"/>
+      <c r="M42" s="182"/>
+      <c r="N42" s="184"/>
+      <c r="O42" s="184"/>
+      <c r="P42" s="184"/>
+      <c r="Q42" s="184"/>
+      <c r="R42" s="184"/>
+      <c r="S42" s="216"/>
+      <c r="T42" s="180"/>
+      <c r="U42" s="180"/>
+      <c r="V42" s="179"/>
+      <c r="W42" s="188"/>
       <c r="Y42" s="28"/>
       <c r="Z42" s="29"/>
       <c r="AA42" s="29"/>
     </row>
     <row r="43" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="203"/>
-      <c r="C43" s="203"/>
-      <c r="D43" s="202"/>
+      <c r="B43" s="207"/>
+      <c r="C43" s="207"/>
+      <c r="D43" s="209"/>
       <c r="F43" s="89"/>
       <c r="G43" s="88"/>
       <c r="H43" s="88"/>
-      <c r="I43" s="208"/>
-      <c r="J43" s="174"/>
-      <c r="K43" s="174"/>
-      <c r="L43" s="174"/>
-      <c r="M43" s="174"/>
-      <c r="N43" s="199"/>
-      <c r="O43" s="199"/>
-      <c r="P43" s="199"/>
-      <c r="Q43" s="199"/>
-      <c r="R43" s="199"/>
-      <c r="S43" s="179"/>
-      <c r="T43" s="182"/>
-      <c r="U43" s="182"/>
-      <c r="V43" s="181"/>
-      <c r="W43" s="193"/>
+      <c r="I43" s="211"/>
+      <c r="J43" s="182"/>
+      <c r="K43" s="182"/>
+      <c r="L43" s="182"/>
+      <c r="M43" s="182"/>
+      <c r="N43" s="184"/>
+      <c r="O43" s="184"/>
+      <c r="P43" s="184"/>
+      <c r="Q43" s="184"/>
+      <c r="R43" s="184"/>
+      <c r="S43" s="216"/>
+      <c r="T43" s="180"/>
+      <c r="U43" s="180"/>
+      <c r="V43" s="179"/>
+      <c r="W43" s="188"/>
       <c r="Y43" s="28"/>
       <c r="Z43" s="29"/>
       <c r="AA43" s="29"/>
     </row>
     <row r="44" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="203"/>
-      <c r="C44" s="203"/>
-      <c r="D44" s="202"/>
+      <c r="B44" s="207"/>
+      <c r="C44" s="207"/>
+      <c r="D44" s="209"/>
       <c r="F44" s="90"/>
       <c r="G44" s="88"/>
       <c r="H44" s="88"/>
-      <c r="I44" s="208"/>
-      <c r="J44" s="174"/>
-      <c r="K44" s="174"/>
-      <c r="L44" s="174"/>
-      <c r="M44" s="174"/>
-      <c r="N44" s="199"/>
-      <c r="O44" s="199"/>
-      <c r="P44" s="199"/>
-      <c r="Q44" s="199"/>
-      <c r="R44" s="199"/>
-      <c r="S44" s="179"/>
-      <c r="T44" s="182"/>
-      <c r="U44" s="182"/>
-      <c r="V44" s="181"/>
-      <c r="W44" s="193"/>
+      <c r="I44" s="211"/>
+      <c r="J44" s="182"/>
+      <c r="K44" s="182"/>
+      <c r="L44" s="182"/>
+      <c r="M44" s="182"/>
+      <c r="N44" s="184"/>
+      <c r="O44" s="184"/>
+      <c r="P44" s="184"/>
+      <c r="Q44" s="184"/>
+      <c r="R44" s="184"/>
+      <c r="S44" s="216"/>
+      <c r="T44" s="180"/>
+      <c r="U44" s="180"/>
+      <c r="V44" s="179"/>
+      <c r="W44" s="188"/>
       <c r="Z44" s="29"/>
       <c r="AA44" s="29"/>
     </row>
     <row r="45" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B45" s="203"/>
-      <c r="C45" s="203"/>
-      <c r="D45" s="202"/>
+      <c r="B45" s="207"/>
+      <c r="C45" s="207"/>
+      <c r="D45" s="209"/>
       <c r="F45" s="87"/>
       <c r="G45" s="88"/>
       <c r="H45" s="88"/>
-      <c r="I45" s="208"/>
-      <c r="J45" s="174"/>
-      <c r="K45" s="174"/>
-      <c r="L45" s="174"/>
-      <c r="M45" s="174"/>
-      <c r="N45" s="199"/>
-      <c r="O45" s="199"/>
-      <c r="P45" s="199"/>
-      <c r="Q45" s="199"/>
-      <c r="R45" s="199"/>
-      <c r="S45" s="179"/>
-      <c r="T45" s="182"/>
-      <c r="U45" s="182"/>
-      <c r="V45" s="181"/>
-      <c r="W45" s="193"/>
+      <c r="I45" s="211"/>
+      <c r="J45" s="182"/>
+      <c r="K45" s="182"/>
+      <c r="L45" s="182"/>
+      <c r="M45" s="182"/>
+      <c r="N45" s="184"/>
+      <c r="O45" s="184"/>
+      <c r="P45" s="184"/>
+      <c r="Q45" s="184"/>
+      <c r="R45" s="184"/>
+      <c r="S45" s="216"/>
+      <c r="T45" s="180"/>
+      <c r="U45" s="180"/>
+      <c r="V45" s="179"/>
+      <c r="W45" s="188"/>
       <c r="Z45" s="29"/>
       <c r="AA45" s="29"/>
     </row>
     <row r="46" spans="2:27" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="203"/>
-      <c r="C46" s="203"/>
-      <c r="D46" s="202"/>
+      <c r="B46" s="207"/>
+      <c r="C46" s="207"/>
+      <c r="D46" s="209"/>
       <c r="F46" s="91"/>
       <c r="G46" s="88"/>
       <c r="H46" s="88"/>
-      <c r="I46" s="209"/>
-      <c r="J46" s="175"/>
-      <c r="K46" s="175"/>
-      <c r="L46" s="175"/>
-      <c r="M46" s="175"/>
-      <c r="N46" s="200"/>
-      <c r="O46" s="200"/>
-      <c r="P46" s="200"/>
-      <c r="Q46" s="200"/>
-      <c r="R46" s="200"/>
-      <c r="S46" s="180"/>
-      <c r="T46" s="183"/>
-      <c r="U46" s="183"/>
-      <c r="V46" s="191"/>
-      <c r="W46" s="194"/>
+      <c r="I46" s="212"/>
+      <c r="J46" s="183"/>
+      <c r="K46" s="183"/>
+      <c r="L46" s="183"/>
+      <c r="M46" s="183"/>
+      <c r="N46" s="185"/>
+      <c r="O46" s="185"/>
+      <c r="P46" s="185"/>
+      <c r="Q46" s="185"/>
+      <c r="R46" s="185"/>
+      <c r="S46" s="217"/>
+      <c r="T46" s="181"/>
+      <c r="U46" s="181"/>
+      <c r="V46" s="186"/>
+      <c r="W46" s="189"/>
       <c r="Z46" s="2"/>
       <c r="AA46" s="2"/>
     </row>
     <row r="47" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B47" s="203"/>
-      <c r="C47" s="203"/>
-      <c r="D47" s="202"/>
+      <c r="B47" s="207"/>
+      <c r="C47" s="207"/>
+      <c r="D47" s="209"/>
       <c r="F47" s="91"/>
       <c r="G47" s="91"/>
       <c r="H47" s="91"/>
@@ -5444,15 +5438,15 @@
       <c r="U47" s="93"/>
       <c r="V47" s="93"/>
       <c r="W47" s="94"/>
-      <c r="Z47" s="184" t="s">
+      <c r="Z47" s="190" t="s">
         <v>6</v>
       </c>
-      <c r="AA47" s="184"/>
+      <c r="AA47" s="190"/>
     </row>
     <row r="48" spans="2:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="203"/>
-      <c r="C48" s="203"/>
-      <c r="D48" s="202"/>
+      <c r="B48" s="207"/>
+      <c r="C48" s="207"/>
+      <c r="D48" s="209"/>
       <c r="E48" s="95"/>
       <c r="F48" s="91"/>
       <c r="G48" s="89"/>
@@ -5483,9 +5477,9 @@
       </c>
     </row>
     <row r="49" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="203"/>
-      <c r="C49" s="203"/>
-      <c r="D49" s="202"/>
+      <c r="B49" s="207"/>
+      <c r="C49" s="207"/>
+      <c r="D49" s="209"/>
       <c r="F49" s="87"/>
       <c r="G49" s="89"/>
       <c r="H49" s="89"/>
@@ -5511,9 +5505,9 @@
       <c r="AA49" s="101"/>
     </row>
     <row r="50" spans="2:27" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B50" s="203"/>
-      <c r="C50" s="203"/>
-      <c r="D50" s="202"/>
+      <c r="B50" s="207"/>
+      <c r="C50" s="207"/>
+      <c r="D50" s="209"/>
       <c r="F50" s="87"/>
       <c r="G50" s="89"/>
       <c r="H50" s="102"/>
@@ -5539,9 +5533,9 @@
       <c r="AA50" s="103"/>
     </row>
     <row r="51" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B51" s="203"/>
-      <c r="C51" s="203"/>
-      <c r="D51" s="202"/>
+      <c r="B51" s="207"/>
+      <c r="C51" s="207"/>
+      <c r="D51" s="209"/>
       <c r="F51" s="87"/>
       <c r="G51" s="87"/>
       <c r="H51" s="87"/>
@@ -5567,9 +5561,9 @@
       <c r="AA51" s="101"/>
     </row>
     <row r="52" spans="2:27" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B52" s="203"/>
-      <c r="C52" s="203"/>
-      <c r="D52" s="202"/>
+      <c r="B52" s="207"/>
+      <c r="C52" s="207"/>
+      <c r="D52" s="209"/>
       <c r="F52" s="104"/>
       <c r="I52" s="96"/>
       <c r="J52" s="97"/>
@@ -5589,9 +5583,9 @@
       <c r="Z52" s="105"/>
     </row>
     <row r="53" spans="2:27" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="203"/>
-      <c r="C53" s="203"/>
-      <c r="D53" s="202"/>
+      <c r="B53" s="207"/>
+      <c r="C53" s="207"/>
+      <c r="D53" s="209"/>
       <c r="E53" s="106"/>
       <c r="F53" s="106"/>
       <c r="G53" s="106"/>
@@ -5615,100 +5609,100 @@
       <c r="AA53" s="105"/>
     </row>
     <row r="54" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B54" s="203"/>
-      <c r="C54" s="203"/>
-      <c r="D54" s="202"/>
-      <c r="E54" s="185"/>
-      <c r="F54" s="185"/>
-      <c r="G54" s="185"/>
-      <c r="H54" s="185"/>
-      <c r="I54" s="185"/>
-      <c r="J54" s="185"/>
-      <c r="K54" s="185"/>
-      <c r="L54" s="185"/>
-      <c r="M54" s="185"/>
-      <c r="N54" s="185"/>
-      <c r="O54" s="185"/>
-      <c r="P54" s="185"/>
-      <c r="Q54" s="185"/>
-      <c r="R54" s="185"/>
-      <c r="S54" s="185"/>
-      <c r="T54" s="185"/>
-      <c r="U54" s="185"/>
-      <c r="V54" s="185"/>
-      <c r="W54" s="186"/>
+      <c r="B54" s="207"/>
+      <c r="C54" s="207"/>
+      <c r="D54" s="209"/>
+      <c r="E54" s="191"/>
+      <c r="F54" s="191"/>
+      <c r="G54" s="191"/>
+      <c r="H54" s="191"/>
+      <c r="I54" s="191"/>
+      <c r="J54" s="191"/>
+      <c r="K54" s="191"/>
+      <c r="L54" s="191"/>
+      <c r="M54" s="191"/>
+      <c r="N54" s="191"/>
+      <c r="O54" s="191"/>
+      <c r="P54" s="191"/>
+      <c r="Q54" s="191"/>
+      <c r="R54" s="191"/>
+      <c r="S54" s="191"/>
+      <c r="T54" s="191"/>
+      <c r="U54" s="191"/>
+      <c r="V54" s="191"/>
+      <c r="W54" s="192"/>
     </row>
     <row r="55" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B55" s="203"/>
-      <c r="C55" s="203"/>
-      <c r="D55" s="202"/>
-      <c r="E55" s="187"/>
-      <c r="F55" s="187"/>
-      <c r="G55" s="187"/>
-      <c r="H55" s="187"/>
-      <c r="I55" s="187"/>
-      <c r="J55" s="187"/>
-      <c r="K55" s="187"/>
-      <c r="L55" s="187"/>
-      <c r="M55" s="187"/>
-      <c r="N55" s="187"/>
-      <c r="O55" s="187"/>
-      <c r="P55" s="187"/>
-      <c r="Q55" s="187"/>
-      <c r="R55" s="187"/>
-      <c r="S55" s="187"/>
-      <c r="T55" s="187"/>
-      <c r="U55" s="187"/>
-      <c r="V55" s="187"/>
-      <c r="W55" s="188"/>
+      <c r="B55" s="207"/>
+      <c r="C55" s="207"/>
+      <c r="D55" s="209"/>
+      <c r="E55" s="172"/>
+      <c r="F55" s="172"/>
+      <c r="G55" s="172"/>
+      <c r="H55" s="172"/>
+      <c r="I55" s="172"/>
+      <c r="J55" s="172"/>
+      <c r="K55" s="172"/>
+      <c r="L55" s="172"/>
+      <c r="M55" s="172"/>
+      <c r="N55" s="172"/>
+      <c r="O55" s="172"/>
+      <c r="P55" s="172"/>
+      <c r="Q55" s="172"/>
+      <c r="R55" s="172"/>
+      <c r="S55" s="172"/>
+      <c r="T55" s="172"/>
+      <c r="U55" s="172"/>
+      <c r="V55" s="172"/>
+      <c r="W55" s="173"/>
     </row>
     <row r="56" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B56" s="203"/>
-      <c r="C56" s="203"/>
-      <c r="D56" s="202"/>
-      <c r="E56" s="187"/>
-      <c r="F56" s="187"/>
-      <c r="G56" s="187"/>
-      <c r="H56" s="187"/>
-      <c r="I56" s="187"/>
-      <c r="J56" s="187"/>
-      <c r="K56" s="187"/>
-      <c r="L56" s="187"/>
-      <c r="M56" s="187"/>
-      <c r="N56" s="187"/>
-      <c r="O56" s="187"/>
-      <c r="P56" s="187"/>
-      <c r="Q56" s="187"/>
-      <c r="R56" s="187"/>
-      <c r="S56" s="187"/>
-      <c r="T56" s="187"/>
-      <c r="U56" s="187"/>
-      <c r="V56" s="187"/>
-      <c r="W56" s="188"/>
+      <c r="B56" s="207"/>
+      <c r="C56" s="207"/>
+      <c r="D56" s="209"/>
+      <c r="E56" s="172"/>
+      <c r="F56" s="172"/>
+      <c r="G56" s="172"/>
+      <c r="H56" s="172"/>
+      <c r="I56" s="172"/>
+      <c r="J56" s="172"/>
+      <c r="K56" s="172"/>
+      <c r="L56" s="172"/>
+      <c r="M56" s="172"/>
+      <c r="N56" s="172"/>
+      <c r="O56" s="172"/>
+      <c r="P56" s="172"/>
+      <c r="Q56" s="172"/>
+      <c r="R56" s="172"/>
+      <c r="S56" s="172"/>
+      <c r="T56" s="172"/>
+      <c r="U56" s="172"/>
+      <c r="V56" s="172"/>
+      <c r="W56" s="173"/>
     </row>
     <row r="57" spans="2:27" ht="64.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="204"/>
-      <c r="C57" s="204"/>
-      <c r="D57" s="205"/>
-      <c r="E57" s="176"/>
-      <c r="F57" s="176"/>
-      <c r="G57" s="176"/>
-      <c r="H57" s="176"/>
-      <c r="I57" s="176"/>
-      <c r="J57" s="176"/>
-      <c r="K57" s="176"/>
-      <c r="L57" s="176"/>
-      <c r="M57" s="176"/>
-      <c r="N57" s="176"/>
-      <c r="O57" s="176"/>
-      <c r="P57" s="176"/>
-      <c r="Q57" s="176"/>
-      <c r="R57" s="176"/>
-      <c r="S57" s="176"/>
-      <c r="T57" s="176"/>
-      <c r="U57" s="176"/>
-      <c r="V57" s="176"/>
-      <c r="W57" s="177"/>
+      <c r="B57" s="208"/>
+      <c r="C57" s="208"/>
+      <c r="D57" s="210"/>
+      <c r="E57" s="213"/>
+      <c r="F57" s="213"/>
+      <c r="G57" s="213"/>
+      <c r="H57" s="213"/>
+      <c r="I57" s="213"/>
+      <c r="J57" s="213"/>
+      <c r="K57" s="213"/>
+      <c r="L57" s="213"/>
+      <c r="M57" s="213"/>
+      <c r="N57" s="213"/>
+      <c r="O57" s="213"/>
+      <c r="P57" s="213"/>
+      <c r="Q57" s="213"/>
+      <c r="R57" s="213"/>
+      <c r="S57" s="213"/>
+      <c r="T57" s="213"/>
+      <c r="U57" s="213"/>
+      <c r="V57" s="213"/>
+      <c r="W57" s="214"/>
     </row>
     <row r="59" spans="2:27" x14ac:dyDescent="0.2">
       <c r="K59" s="110" t="s">
@@ -5730,10 +5724,10 @@
       <c r="S59" s="119" t="s">
         <v>15</v>
       </c>
-      <c r="T59" s="189" t="s">
+      <c r="T59" s="177" t="s">
         <v>21</v>
       </c>
-      <c r="U59" s="190"/>
+      <c r="U59" s="178"/>
       <c r="V59" s="111"/>
       <c r="W59" s="111"/>
       <c r="X59" s="111"/>
@@ -5764,10 +5758,10 @@
       <c r="S60" s="132" t="s">
         <v>16</v>
       </c>
-      <c r="T60" s="189" t="s">
+      <c r="T60" s="177" t="s">
         <v>22</v>
       </c>
-      <c r="U60" s="190"/>
+      <c r="U60" s="178"/>
       <c r="V60" s="113"/>
       <c r="W60" s="113"/>
       <c r="X60" s="113"/>
@@ -5779,10 +5773,10 @@
       <c r="S61" s="142" t="s">
         <v>17</v>
       </c>
-      <c r="T61" s="189" t="s">
+      <c r="T61" s="177" t="s">
         <v>23</v>
       </c>
-      <c r="U61" s="190"/>
+      <c r="U61" s="178"/>
       <c r="Y61" s="1"/>
       <c r="Z61" s="1"/>
       <c r="AA61" s="1"/>
@@ -5812,50 +5806,6 @@
     </row>
   </sheetData>
   <mergeCells count="60">
-    <mergeCell ref="F34:H34"/>
-    <mergeCell ref="F36:H36"/>
-    <mergeCell ref="F37:H37"/>
-    <mergeCell ref="F35:H35"/>
-    <mergeCell ref="F28:H28"/>
-    <mergeCell ref="F29:H29"/>
-    <mergeCell ref="F30:H30"/>
-    <mergeCell ref="F33:H33"/>
-    <mergeCell ref="F23:H23"/>
-    <mergeCell ref="F24:H24"/>
-    <mergeCell ref="F25:H25"/>
-    <mergeCell ref="F26:H26"/>
-    <mergeCell ref="F27:H27"/>
-    <mergeCell ref="F18:H18"/>
-    <mergeCell ref="F19:H19"/>
-    <mergeCell ref="F20:H20"/>
-    <mergeCell ref="F21:H21"/>
-    <mergeCell ref="F22:H22"/>
-    <mergeCell ref="F13:H13"/>
-    <mergeCell ref="F14:H14"/>
-    <mergeCell ref="F15:H15"/>
-    <mergeCell ref="F16:H16"/>
-    <mergeCell ref="F17:H17"/>
-    <mergeCell ref="F8:H8"/>
-    <mergeCell ref="F9:H9"/>
-    <mergeCell ref="F10:H10"/>
-    <mergeCell ref="F11:H11"/>
-    <mergeCell ref="F12:H12"/>
-    <mergeCell ref="T61:U61"/>
-    <mergeCell ref="E56:W56"/>
-    <mergeCell ref="U41:U46"/>
-    <mergeCell ref="L41:L46"/>
-    <mergeCell ref="M41:M46"/>
-    <mergeCell ref="N41:N46"/>
-    <mergeCell ref="O41:O46"/>
-    <mergeCell ref="P41:P46"/>
-    <mergeCell ref="Q41:Q46"/>
-    <mergeCell ref="V41:V46"/>
-    <mergeCell ref="W41:W46"/>
-    <mergeCell ref="Z47:AA47"/>
-    <mergeCell ref="E54:W54"/>
-    <mergeCell ref="E55:W55"/>
-    <mergeCell ref="T59:U59"/>
-    <mergeCell ref="T60:U60"/>
     <mergeCell ref="E3:W4"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="I5:R5"/>
@@ -5872,6 +5822,50 @@
     <mergeCell ref="T41:T46"/>
     <mergeCell ref="F6:H6"/>
     <mergeCell ref="F7:H7"/>
+    <mergeCell ref="Z47:AA47"/>
+    <mergeCell ref="E54:W54"/>
+    <mergeCell ref="E55:W55"/>
+    <mergeCell ref="T59:U59"/>
+    <mergeCell ref="T60:U60"/>
+    <mergeCell ref="T61:U61"/>
+    <mergeCell ref="E56:W56"/>
+    <mergeCell ref="U41:U46"/>
+    <mergeCell ref="L41:L46"/>
+    <mergeCell ref="M41:M46"/>
+    <mergeCell ref="N41:N46"/>
+    <mergeCell ref="O41:O46"/>
+    <mergeCell ref="P41:P46"/>
+    <mergeCell ref="Q41:Q46"/>
+    <mergeCell ref="V41:V46"/>
+    <mergeCell ref="W41:W46"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="F9:H9"/>
+    <mergeCell ref="F10:H10"/>
+    <mergeCell ref="F11:H11"/>
+    <mergeCell ref="F12:H12"/>
+    <mergeCell ref="F13:H13"/>
+    <mergeCell ref="F14:H14"/>
+    <mergeCell ref="F15:H15"/>
+    <mergeCell ref="F16:H16"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="F18:H18"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="F21:H21"/>
+    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="F24:H24"/>
+    <mergeCell ref="F25:H25"/>
+    <mergeCell ref="F26:H26"/>
+    <mergeCell ref="F27:H27"/>
+    <mergeCell ref="F34:H34"/>
+    <mergeCell ref="F36:H36"/>
+    <mergeCell ref="F37:H37"/>
+    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="F28:H28"/>
+    <mergeCell ref="F29:H29"/>
+    <mergeCell ref="F30:H30"/>
+    <mergeCell ref="F33:H33"/>
   </mergeCells>
   <conditionalFormatting sqref="B40:D40">
     <cfRule type="cellIs" dxfId="22" priority="58" stopIfTrue="1" operator="notEqual">
@@ -5889,33 +5883,33 @@
       <formula>"R"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I20:L27 I16:R19 J6:R6 I7:I8 K7:R8 I9:J9 L9:R9 I10:K10 M10:R10 I11:L11 N11:R11 I12:M12 O12:R12 I13:N13 P13:R13 I14:O14 Q14:R14 I15:P15 R15">
-    <cfRule type="cellIs" dxfId="18" priority="49" stopIfTrue="1" operator="equal">
-      <formula>"S"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="17" priority="50" stopIfTrue="1" operator="equal">
-      <formula>"C"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="51" stopIfTrue="1" operator="equal">
-      <formula>"D"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="I30:R39">
-    <cfRule type="cellIs" dxfId="15" priority="12" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="12" stopIfTrue="1" operator="equal">
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I30:R40">
-    <cfRule type="cellIs" dxfId="14" priority="10" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="10" stopIfTrue="1" operator="equal">
       <formula>"S"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="11" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="11" stopIfTrue="1" operator="equal">
       <formula>"C"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I40:R40">
-    <cfRule type="cellIs" dxfId="12" priority="61" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="61" stopIfTrue="1" operator="equal">
       <formula>"L"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J6:R6 I7:I8 K7:R8 I9:J9 L9:R9 I10:K10 M10:R10 I11:L11 N11:R11 I12:M12 O12:R12 I13:N13 P13:R13 I14:O14 Q14:R14 I15:P15 R15 I16:R19 I20:L27">
+    <cfRule type="cellIs" dxfId="14" priority="49" stopIfTrue="1" operator="equal">
+      <formula>"S"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="13" priority="50" stopIfTrue="1" operator="equal">
+      <formula>"C"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="51" stopIfTrue="1" operator="equal">
+      <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M20:P25 R20:R29 N26:P27 I28:P28 I29:O29 Q29">

</xml_diff>

<commit_message>
update docs, removing waste, bug fix, add tests
</commit_message>
<xml_diff>
--- a/Task 2/OPPM_Plan.xlsx
+++ b/Task 2/OPPM_Plan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kohaku\Downloads\LAB301\Task 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC7DB633-2284-4261-BC2E-03E1593735D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6A46908-08B0-41C3-A036-E922A3124B06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start" sheetId="2" r:id="rId1"/>
@@ -30,20 +30,11 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={3486CE5B-0EEB-4ADC-B63E-BB85D4F28BAC}</author>
     <author>tc={216EE87A-CE1B-41F5-8655-E24D6D9DB930}</author>
     <author>Microsoft Office User</author>
   </authors>
   <commentList>
-    <comment ref="O13" authorId="0" shapeId="0" xr:uid="{3486CE5B-0EEB-4ADC-B63E-BB85D4F28BAC}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    This is basically just a buffer for func 1 2 3 since we are not doing func 4</t>
-      </text>
-    </comment>
-    <comment ref="Y47" authorId="1" shapeId="0" xr:uid="{216EE87A-CE1B-41F5-8655-E24D6D9DB930}">
+    <comment ref="Y47" authorId="0" shapeId="0" xr:uid="{216EE87A-CE1B-41F5-8655-E24D6D9DB930}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -52,7 +43,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="J60" authorId="2" shapeId="0" xr:uid="{F90B73BB-1F15-CD43-AECB-A57B7C17353B}">
+    <comment ref="J60" authorId="1" shapeId="0" xr:uid="{F90B73BB-1F15-CD43-AECB-A57B7C17353B}">
       <text>
         <r>
           <rPr>
@@ -2042,6 +2033,172 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="55" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="55" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="48" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="67" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="66" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="4" fillId="8" borderId="55" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="4" fillId="8" borderId="48" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="4" fillId="0" borderId="55" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="4" fillId="0" borderId="48" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="59" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="4" fillId="0" borderId="72" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="4" fillId="0" borderId="73" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="55" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="55" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="48" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="49" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="68" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="63" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="49" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="50" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
       <protection locked="0"/>
@@ -2066,18 +2223,6 @@
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="69" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
       <protection locked="0"/>
@@ -2088,160 +2233,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="71" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="63" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="49" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="4" fillId="0" borderId="55" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="4" fillId="0" borderId="48" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="4" fillId="0" borderId="72" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="4" fillId="0" borderId="73" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="49" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="50" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="55" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="55" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="48" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="67" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="66" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="4" fillId="8" borderId="55" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="4" fillId="8" borderId="48" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="59" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="55" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="55" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="48" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="68" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -2912,7 +2903,7 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:noFill/>
             </a14:hiddenFill>
           </a:ext>
@@ -2966,7 +2957,7 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:noFill/>
             </a14:hiddenFill>
           </a:ext>
@@ -3322,14 +3313,14 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="3175">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="3175">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -3388,7 +3379,7 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:noFill/>
             </a14:hiddenFill>
           </a:ext>
@@ -3442,7 +3433,7 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:noFill/>
             </a14:hiddenFill>
           </a:ext>
@@ -3496,7 +3487,7 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:noFill/>
             </a14:hiddenFill>
           </a:ext>
@@ -3993,9 +3984,6 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="O13" dT="2026-06-15T09:00:51.90" personId="{EB96A237-E87F-443C-9291-CBF6B404B456}" id="{3486CE5B-0EEB-4ADC-B63E-BB85D4F28BAC}">
-    <text>This is basically just a buffer for func 1 2 3 since we are not doing func 4</text>
-  </threadedComment>
   <threadedComment ref="Y47" dT="2026-06-15T09:01:16.29" personId="{EB96A237-E87F-443C-9291-CBF6B404B456}" id="{216EE87A-CE1B-41F5-8655-E24D6D9DB930}">
     <text xml:space="preserve">Do I  need to fill these ?
 </text>
@@ -4009,25 +3997,25 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:AA65"/>
-  <sheetFormatPr defaultColWidth="10.125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.08203125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" style="1" customWidth="1"/>
-    <col min="2" max="5" width="3.875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="21.125" style="1" customWidth="1"/>
+    <col min="2" max="5" width="3.83203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="21.08203125" style="1" customWidth="1"/>
     <col min="7" max="7" width="25" style="1" customWidth="1"/>
-    <col min="8" max="8" width="11.375" style="1" customWidth="1"/>
-    <col min="9" max="18" width="5.875" style="1" customWidth="1"/>
-    <col min="19" max="22" width="4.875" style="1" customWidth="1"/>
-    <col min="23" max="23" width="5.125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="11.33203125" style="1" customWidth="1"/>
+    <col min="9" max="18" width="5.83203125" style="1" customWidth="1"/>
+    <col min="19" max="22" width="4.83203125" style="1" customWidth="1"/>
+    <col min="23" max="23" width="5.08203125" style="1" customWidth="1"/>
     <col min="24" max="24" width="3" style="1" customWidth="1"/>
-    <col min="25" max="25" width="15.375" style="2" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="9.125" style="3" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="9.625" style="3" bestFit="1" customWidth="1"/>
-    <col min="28" max="16384" width="10.125" style="1"/>
+    <col min="25" max="25" width="15.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="9.08203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="9.58203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="28" max="16384" width="10.08203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:27" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:27" s="4" customFormat="1" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:27" ht="13" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:27" s="4" customFormat="1" ht="18" x14ac:dyDescent="0.4">
       <c r="B2" s="5"/>
       <c r="C2" s="6"/>
       <c r="D2" s="7"/>
@@ -4060,94 +4048,94 @@
       <c r="Z2" s="13"/>
       <c r="AA2" s="13"/>
     </row>
-    <row r="3" spans="2:27" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:27" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B3" s="14"/>
       <c r="D3" s="15"/>
-      <c r="E3" s="193" t="s">
+      <c r="E3" s="165" t="s">
         <v>31</v>
       </c>
-      <c r="F3" s="194"/>
-      <c r="G3" s="194"/>
-      <c r="H3" s="194"/>
-      <c r="I3" s="194"/>
-      <c r="J3" s="194"/>
-      <c r="K3" s="194"/>
-      <c r="L3" s="194"/>
-      <c r="M3" s="194"/>
-      <c r="N3" s="194"/>
-      <c r="O3" s="194"/>
-      <c r="P3" s="194"/>
-      <c r="Q3" s="194"/>
-      <c r="R3" s="194"/>
-      <c r="S3" s="194"/>
-      <c r="T3" s="194"/>
-      <c r="U3" s="194"/>
-      <c r="V3" s="194"/>
-      <c r="W3" s="195"/>
+      <c r="F3" s="166"/>
+      <c r="G3" s="166"/>
+      <c r="H3" s="166"/>
+      <c r="I3" s="166"/>
+      <c r="J3" s="166"/>
+      <c r="K3" s="166"/>
+      <c r="L3" s="166"/>
+      <c r="M3" s="166"/>
+      <c r="N3" s="166"/>
+      <c r="O3" s="166"/>
+      <c r="P3" s="166"/>
+      <c r="Q3" s="166"/>
+      <c r="R3" s="166"/>
+      <c r="S3" s="166"/>
+      <c r="T3" s="166"/>
+      <c r="U3" s="166"/>
+      <c r="V3" s="166"/>
+      <c r="W3" s="167"/>
       <c r="Y3" s="12"/>
       <c r="Z3" s="13"/>
       <c r="AA3" s="13"/>
     </row>
-    <row r="4" spans="2:27" s="16" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:27" s="16" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B4" s="17"/>
       <c r="C4" s="18"/>
       <c r="D4" s="18"/>
-      <c r="E4" s="196"/>
-      <c r="F4" s="197"/>
-      <c r="G4" s="197"/>
-      <c r="H4" s="197"/>
-      <c r="I4" s="197"/>
-      <c r="J4" s="197"/>
-      <c r="K4" s="197"/>
-      <c r="L4" s="197"/>
-      <c r="M4" s="197"/>
-      <c r="N4" s="197"/>
-      <c r="O4" s="197"/>
-      <c r="P4" s="197"/>
-      <c r="Q4" s="197"/>
-      <c r="R4" s="197"/>
-      <c r="S4" s="197"/>
-      <c r="T4" s="197"/>
-      <c r="U4" s="197"/>
-      <c r="V4" s="197"/>
-      <c r="W4" s="198"/>
+      <c r="E4" s="168"/>
+      <c r="F4" s="169"/>
+      <c r="G4" s="169"/>
+      <c r="H4" s="169"/>
+      <c r="I4" s="169"/>
+      <c r="J4" s="169"/>
+      <c r="K4" s="169"/>
+      <c r="L4" s="169"/>
+      <c r="M4" s="169"/>
+      <c r="N4" s="169"/>
+      <c r="O4" s="169"/>
+      <c r="P4" s="169"/>
+      <c r="Q4" s="169"/>
+      <c r="R4" s="169"/>
+      <c r="S4" s="169"/>
+      <c r="T4" s="169"/>
+      <c r="U4" s="169"/>
+      <c r="V4" s="169"/>
+      <c r="W4" s="170"/>
       <c r="Y4" s="19"/>
       <c r="Z4" s="20"/>
       <c r="AA4" s="20"/>
     </row>
-    <row r="5" spans="2:27" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="199" t="s">
+    <row r="5" spans="2:27" ht="14" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="171" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="200"/>
-      <c r="D5" s="201"/>
+      <c r="C5" s="172"/>
+      <c r="D5" s="173"/>
       <c r="E5" s="21"/>
       <c r="F5" s="22" t="s">
         <v>1</v>
       </c>
       <c r="G5" s="23"/>
       <c r="H5" s="23"/>
-      <c r="I5" s="202" t="s">
+      <c r="I5" s="174" t="s">
         <v>2</v>
       </c>
-      <c r="J5" s="203"/>
-      <c r="K5" s="203"/>
-      <c r="L5" s="203"/>
-      <c r="M5" s="203"/>
-      <c r="N5" s="203"/>
-      <c r="O5" s="203"/>
-      <c r="P5" s="203"/>
-      <c r="Q5" s="203"/>
-      <c r="R5" s="204"/>
-      <c r="S5" s="202" t="s">
+      <c r="J5" s="175"/>
+      <c r="K5" s="175"/>
+      <c r="L5" s="175"/>
+      <c r="M5" s="175"/>
+      <c r="N5" s="175"/>
+      <c r="O5" s="175"/>
+      <c r="P5" s="175"/>
+      <c r="Q5" s="175"/>
+      <c r="R5" s="176"/>
+      <c r="S5" s="174" t="s">
         <v>3</v>
       </c>
-      <c r="T5" s="203"/>
-      <c r="U5" s="203"/>
-      <c r="V5" s="204"/>
-      <c r="W5" s="205"/>
-    </row>
-    <row r="6" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="T5" s="175"/>
+      <c r="U5" s="175"/>
+      <c r="V5" s="176"/>
+      <c r="W5" s="177"/>
+    </row>
+    <row r="6" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="25"/>
       <c r="C6" s="26"/>
       <c r="D6" s="112" t="s">
@@ -4156,11 +4144,11 @@
       <c r="E6" s="114">
         <v>1</v>
       </c>
-      <c r="F6" s="218" t="s">
+      <c r="F6" s="197" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="191"/>
-      <c r="H6" s="192"/>
+      <c r="G6" s="198"/>
+      <c r="H6" s="199"/>
       <c r="I6" s="112" t="s">
         <v>10</v>
       </c>
@@ -4184,7 +4172,7 @@
       <c r="Z6" s="29"/>
       <c r="AA6" s="29"/>
     </row>
-    <row r="7" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="25"/>
       <c r="C7" s="54"/>
       <c r="D7" s="112" t="s">
@@ -4193,11 +4181,11 @@
       <c r="E7" s="125">
         <v>2</v>
       </c>
-      <c r="F7" s="171" t="s">
+      <c r="F7" s="200" t="s">
         <v>34</v>
       </c>
-      <c r="G7" s="172"/>
-      <c r="H7" s="173"/>
+      <c r="G7" s="201"/>
+      <c r="H7" s="202"/>
       <c r="I7" s="137"/>
       <c r="J7" s="112" t="s">
         <v>10</v>
@@ -4221,7 +4209,7 @@
       <c r="Z7" s="29"/>
       <c r="AA7" s="29"/>
     </row>
-    <row r="8" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="25"/>
       <c r="C8" s="30"/>
       <c r="D8" s="112" t="s">
@@ -4230,11 +4218,11 @@
       <c r="E8" s="115">
         <v>3</v>
       </c>
-      <c r="F8" s="171" t="s">
+      <c r="F8" s="200" t="s">
         <v>35</v>
       </c>
-      <c r="G8" s="172"/>
-      <c r="H8" s="173"/>
+      <c r="G8" s="201"/>
+      <c r="H8" s="202"/>
       <c r="I8" s="32"/>
       <c r="J8" s="112" t="s">
         <v>10</v>
@@ -4257,24 +4245,24 @@
       <c r="Z8" s="29"/>
       <c r="AA8" s="29"/>
     </row>
-    <row r="9" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="25"/>
       <c r="C9" s="30"/>
       <c r="D9" s="112" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E9" s="115">
         <v>4</v>
       </c>
-      <c r="F9" s="171" t="s">
+      <c r="F9" s="200" t="s">
         <v>36</v>
       </c>
-      <c r="G9" s="172"/>
-      <c r="H9" s="173"/>
+      <c r="G9" s="201"/>
+      <c r="H9" s="202"/>
       <c r="I9" s="32"/>
       <c r="J9" s="33"/>
       <c r="K9" s="112" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L9" s="37"/>
       <c r="M9" s="36"/>
@@ -4294,25 +4282,25 @@
       <c r="Z9" s="29"/>
       <c r="AA9" s="29"/>
     </row>
-    <row r="10" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="25"/>
       <c r="C10" s="112" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D10" s="31"/>
       <c r="E10" s="115">
         <v>5</v>
       </c>
-      <c r="F10" s="171" t="s">
+      <c r="F10" s="200" t="s">
         <v>37</v>
       </c>
-      <c r="G10" s="172"/>
-      <c r="H10" s="173"/>
+      <c r="G10" s="201"/>
+      <c r="H10" s="202"/>
       <c r="I10" s="32"/>
       <c r="J10" s="33"/>
       <c r="K10" s="35"/>
       <c r="L10" s="112" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="M10" s="36"/>
       <c r="N10" s="33"/>
@@ -4330,26 +4318,26 @@
       <c r="Z10" s="29"/>
       <c r="AA10" s="29"/>
     </row>
-    <row r="11" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="25"/>
       <c r="C11" s="112" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D11" s="31"/>
       <c r="E11" s="115">
         <v>6</v>
       </c>
-      <c r="F11" s="171" t="s">
+      <c r="F11" s="200" t="s">
         <v>38</v>
       </c>
-      <c r="G11" s="172"/>
-      <c r="H11" s="173"/>
+      <c r="G11" s="201"/>
+      <c r="H11" s="202"/>
       <c r="I11" s="32"/>
       <c r="J11" s="33"/>
       <c r="K11" s="37"/>
       <c r="L11" s="37"/>
       <c r="M11" s="112" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="N11" s="33"/>
       <c r="O11" s="33"/>
@@ -4367,27 +4355,27 @@
       <c r="Z11" s="29"/>
       <c r="AA11" s="29"/>
     </row>
-    <row r="12" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="25"/>
       <c r="C12" s="112" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D12" s="31"/>
       <c r="E12" s="115">
         <v>7</v>
       </c>
-      <c r="F12" s="171" t="s">
+      <c r="F12" s="200" t="s">
         <v>39</v>
       </c>
-      <c r="G12" s="172"/>
-      <c r="H12" s="173"/>
+      <c r="G12" s="201"/>
+      <c r="H12" s="202"/>
       <c r="I12" s="32"/>
       <c r="J12" s="33"/>
       <c r="K12" s="33"/>
       <c r="L12" s="37"/>
       <c r="M12" s="33"/>
       <c r="N12" s="112" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="O12" s="33"/>
       <c r="P12" s="33"/>
@@ -4404,20 +4392,20 @@
       <c r="Z12" s="29"/>
       <c r="AA12" s="29"/>
     </row>
-    <row r="13" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="25" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C13" s="30"/>
       <c r="D13" s="31"/>
       <c r="E13" s="115">
         <v>8</v>
       </c>
-      <c r="F13" s="171" t="s">
+      <c r="F13" s="200" t="s">
         <v>40</v>
       </c>
-      <c r="G13" s="172"/>
-      <c r="H13" s="173"/>
+      <c r="G13" s="201"/>
+      <c r="H13" s="202"/>
       <c r="I13" s="32"/>
       <c r="J13" s="33"/>
       <c r="K13" s="33"/>
@@ -4425,7 +4413,7 @@
       <c r="M13" s="33"/>
       <c r="N13" s="33"/>
       <c r="O13" s="112" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="P13" s="33"/>
       <c r="Q13" s="33"/>
@@ -4441,20 +4429,20 @@
       <c r="Z13" s="29"/>
       <c r="AA13" s="29"/>
     </row>
-    <row r="14" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="25" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C14" s="30"/>
       <c r="D14" s="31"/>
       <c r="E14" s="115">
         <v>9</v>
       </c>
-      <c r="F14" s="171" t="s">
+      <c r="F14" s="200" t="s">
         <v>41</v>
       </c>
-      <c r="G14" s="172"/>
-      <c r="H14" s="173"/>
+      <c r="G14" s="201"/>
+      <c r="H14" s="202"/>
       <c r="I14" s="32"/>
       <c r="J14" s="33"/>
       <c r="K14" s="33"/>
@@ -4463,7 +4451,7 @@
       <c r="N14" s="33"/>
       <c r="O14" s="33"/>
       <c r="P14" s="112" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="Q14" s="33"/>
       <c r="R14" s="33"/>
@@ -4478,7 +4466,7 @@
       <c r="Z14" s="29"/>
       <c r="AA14" s="29"/>
     </row>
-    <row r="15" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="25" t="s">
         <v>11</v>
       </c>
@@ -4487,11 +4475,11 @@
       <c r="E15" s="115">
         <v>10</v>
       </c>
-      <c r="F15" s="171" t="s">
+      <c r="F15" s="200" t="s">
         <v>42</v>
       </c>
-      <c r="G15" s="172"/>
-      <c r="H15" s="173"/>
+      <c r="G15" s="201"/>
+      <c r="H15" s="202"/>
       <c r="I15" s="32"/>
       <c r="J15" s="33"/>
       <c r="K15" s="33"/>
@@ -4515,16 +4503,16 @@
       <c r="Z15" s="29"/>
       <c r="AA15" s="29"/>
     </row>
-    <row r="16" spans="2:27" s="24" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:27" s="24" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="B16" s="25"/>
       <c r="C16" s="30"/>
       <c r="D16" s="31"/>
       <c r="E16" s="115">
         <v>11</v>
       </c>
-      <c r="F16" s="171"/>
-      <c r="G16" s="172"/>
-      <c r="H16" s="173"/>
+      <c r="F16" s="200"/>
+      <c r="G16" s="201"/>
+      <c r="H16" s="202"/>
       <c r="I16" s="32"/>
       <c r="J16" s="33"/>
       <c r="K16" s="33"/>
@@ -4544,16 +4532,16 @@
       <c r="Z16" s="29"/>
       <c r="AA16" s="29"/>
     </row>
-    <row r="17" spans="2:27" s="24" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:27" s="24" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="B17" s="25"/>
       <c r="C17" s="30"/>
       <c r="D17" s="31"/>
       <c r="E17" s="115">
         <v>12</v>
       </c>
-      <c r="F17" s="171"/>
-      <c r="G17" s="172"/>
-      <c r="H17" s="173"/>
+      <c r="F17" s="200"/>
+      <c r="G17" s="201"/>
+      <c r="H17" s="202"/>
       <c r="I17" s="32"/>
       <c r="J17" s="33"/>
       <c r="K17" s="33"/>
@@ -4573,16 +4561,16 @@
       <c r="Z17" s="29"/>
       <c r="AA17" s="29"/>
     </row>
-    <row r="18" spans="2:27" s="24" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:27" s="24" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="B18" s="25"/>
       <c r="C18" s="30"/>
       <c r="D18" s="31"/>
       <c r="E18" s="115">
         <v>13</v>
       </c>
-      <c r="F18" s="171"/>
-      <c r="G18" s="172"/>
-      <c r="H18" s="173"/>
+      <c r="F18" s="200"/>
+      <c r="G18" s="201"/>
+      <c r="H18" s="202"/>
       <c r="I18" s="32"/>
       <c r="J18" s="33"/>
       <c r="K18" s="33"/>
@@ -4601,16 +4589,16 @@
       <c r="Z18" s="29"/>
       <c r="AA18" s="29"/>
     </row>
-    <row r="19" spans="2:27" s="24" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:27" s="24" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="B19" s="25"/>
       <c r="C19" s="30"/>
       <c r="D19" s="31"/>
       <c r="E19" s="115">
         <v>14</v>
       </c>
-      <c r="F19" s="171"/>
-      <c r="G19" s="172"/>
-      <c r="H19" s="173"/>
+      <c r="F19" s="200"/>
+      <c r="G19" s="201"/>
+      <c r="H19" s="202"/>
       <c r="I19" s="32"/>
       <c r="J19" s="33"/>
       <c r="K19" s="33"/>
@@ -4630,16 +4618,16 @@
       <c r="Z19" s="29"/>
       <c r="AA19" s="29"/>
     </row>
-    <row r="20" spans="2:27" s="24" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:27" s="24" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="B20" s="25"/>
       <c r="C20" s="30"/>
       <c r="D20" s="31"/>
       <c r="E20" s="115">
         <v>15</v>
       </c>
-      <c r="F20" s="171"/>
-      <c r="G20" s="172"/>
-      <c r="H20" s="173"/>
+      <c r="F20" s="200"/>
+      <c r="G20" s="201"/>
+      <c r="H20" s="202"/>
       <c r="I20" s="32"/>
       <c r="J20" s="33"/>
       <c r="K20" s="33"/>
@@ -4659,16 +4647,16 @@
       <c r="Z20" s="29"/>
       <c r="AA20" s="29"/>
     </row>
-    <row r="21" spans="2:27" s="24" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:27" s="24" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="B21" s="25"/>
       <c r="C21" s="30"/>
       <c r="D21" s="31"/>
       <c r="E21" s="115">
         <v>16</v>
       </c>
-      <c r="F21" s="171"/>
-      <c r="G21" s="172"/>
-      <c r="H21" s="173"/>
+      <c r="F21" s="200"/>
+      <c r="G21" s="201"/>
+      <c r="H21" s="202"/>
       <c r="I21" s="32"/>
       <c r="J21" s="33"/>
       <c r="K21" s="33"/>
@@ -4688,16 +4676,16 @@
       <c r="Z21" s="29"/>
       <c r="AA21" s="29"/>
     </row>
-    <row r="22" spans="2:27" s="24" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:27" s="24" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="B22" s="25"/>
       <c r="C22" s="30"/>
       <c r="D22" s="31"/>
       <c r="E22" s="115">
         <v>17</v>
       </c>
-      <c r="F22" s="171"/>
-      <c r="G22" s="172"/>
-      <c r="H22" s="173"/>
+      <c r="F22" s="200"/>
+      <c r="G22" s="201"/>
+      <c r="H22" s="202"/>
       <c r="I22" s="32"/>
       <c r="J22" s="33"/>
       <c r="K22" s="33"/>
@@ -4717,16 +4705,16 @@
       <c r="Z22" s="29"/>
       <c r="AA22" s="29"/>
     </row>
-    <row r="23" spans="2:27" s="24" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:27" s="24" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="B23" s="25"/>
       <c r="C23" s="30"/>
       <c r="D23" s="31"/>
       <c r="E23" s="115">
         <v>18</v>
       </c>
-      <c r="F23" s="171"/>
-      <c r="G23" s="172"/>
-      <c r="H23" s="173"/>
+      <c r="F23" s="200"/>
+      <c r="G23" s="201"/>
+      <c r="H23" s="202"/>
       <c r="I23" s="32"/>
       <c r="J23" s="33"/>
       <c r="K23" s="33"/>
@@ -4746,16 +4734,16 @@
       <c r="Z23" s="29"/>
       <c r="AA23" s="29"/>
     </row>
-    <row r="24" spans="2:27" s="24" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:27" s="24" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="B24" s="25"/>
       <c r="C24" s="30"/>
       <c r="D24" s="31"/>
       <c r="E24" s="115">
         <v>19</v>
       </c>
-      <c r="F24" s="171"/>
-      <c r="G24" s="172"/>
-      <c r="H24" s="173"/>
+      <c r="F24" s="200"/>
+      <c r="G24" s="201"/>
+      <c r="H24" s="202"/>
       <c r="I24" s="32"/>
       <c r="J24" s="33"/>
       <c r="K24" s="33"/>
@@ -4774,16 +4762,16 @@
       <c r="Z24" s="29"/>
       <c r="AA24" s="29"/>
     </row>
-    <row r="25" spans="2:27" s="24" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:27" s="24" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="B25" s="25"/>
       <c r="C25" s="30"/>
       <c r="D25" s="31"/>
       <c r="E25" s="115">
         <v>20</v>
       </c>
-      <c r="F25" s="171"/>
-      <c r="G25" s="172"/>
-      <c r="H25" s="173"/>
+      <c r="F25" s="200"/>
+      <c r="G25" s="201"/>
+      <c r="H25" s="202"/>
       <c r="I25" s="32"/>
       <c r="J25" s="33"/>
       <c r="K25" s="33"/>
@@ -4803,16 +4791,16 @@
       <c r="Z25" s="29"/>
       <c r="AA25" s="29"/>
     </row>
-    <row r="26" spans="2:27" s="24" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:27" s="24" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="B26" s="25"/>
       <c r="C26" s="30"/>
       <c r="D26" s="31"/>
       <c r="E26" s="115">
         <v>21</v>
       </c>
-      <c r="F26" s="171"/>
-      <c r="G26" s="172"/>
-      <c r="H26" s="173"/>
+      <c r="F26" s="200"/>
+      <c r="G26" s="201"/>
+      <c r="H26" s="202"/>
       <c r="I26" s="32"/>
       <c r="J26" s="33"/>
       <c r="K26" s="33"/>
@@ -4831,16 +4819,16 @@
       <c r="Z26" s="29"/>
       <c r="AA26" s="29"/>
     </row>
-    <row r="27" spans="2:27" s="24" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:27" s="24" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="B27" s="25"/>
       <c r="C27" s="30"/>
       <c r="D27" s="31"/>
       <c r="E27" s="115">
         <v>22</v>
       </c>
-      <c r="F27" s="171"/>
-      <c r="G27" s="172"/>
-      <c r="H27" s="173"/>
+      <c r="F27" s="200"/>
+      <c r="G27" s="201"/>
+      <c r="H27" s="202"/>
       <c r="I27" s="32"/>
       <c r="J27" s="33"/>
       <c r="K27" s="33"/>
@@ -4860,16 +4848,16 @@
       <c r="Z27" s="29"/>
       <c r="AA27" s="29"/>
     </row>
-    <row r="28" spans="2:27" s="24" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:27" s="24" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="B28" s="25"/>
       <c r="C28" s="30"/>
       <c r="D28" s="31"/>
       <c r="E28" s="115">
         <v>23</v>
       </c>
-      <c r="F28" s="171"/>
-      <c r="G28" s="172"/>
-      <c r="H28" s="173"/>
+      <c r="F28" s="200"/>
+      <c r="G28" s="201"/>
+      <c r="H28" s="202"/>
       <c r="I28" s="32"/>
       <c r="J28" s="33"/>
       <c r="K28" s="33"/>
@@ -4887,16 +4875,16 @@
       <c r="Z28" s="29"/>
       <c r="AA28" s="29"/>
     </row>
-    <row r="29" spans="2:27" s="24" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:27" s="24" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="B29" s="39"/>
       <c r="C29" s="40"/>
       <c r="D29" s="41"/>
       <c r="E29" s="140">
         <v>24</v>
       </c>
-      <c r="F29" s="171"/>
-      <c r="G29" s="172"/>
-      <c r="H29" s="173"/>
+      <c r="F29" s="200"/>
+      <c r="G29" s="201"/>
+      <c r="H29" s="202"/>
       <c r="I29" s="141"/>
       <c r="J29" s="34"/>
       <c r="K29" s="34"/>
@@ -4915,16 +4903,16 @@
       <c r="Z29" s="29"/>
       <c r="AA29" s="29"/>
     </row>
-    <row r="30" spans="2:27" s="24" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:27" s="24" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="B30" s="39"/>
       <c r="C30" s="40"/>
       <c r="D30" s="41"/>
       <c r="E30" s="140">
         <v>25</v>
       </c>
-      <c r="F30" s="171"/>
-      <c r="G30" s="172"/>
-      <c r="H30" s="173"/>
+      <c r="F30" s="200"/>
+      <c r="G30" s="201"/>
+      <c r="H30" s="202"/>
       <c r="I30" s="141"/>
       <c r="J30" s="34"/>
       <c r="K30" s="34"/>
@@ -4944,7 +4932,7 @@
       <c r="Z30" s="29"/>
       <c r="AA30" s="29"/>
     </row>
-    <row r="31" spans="2:27" s="24" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:27" s="24" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="B31" s="39"/>
       <c r="C31" s="40"/>
       <c r="D31" s="41"/>
@@ -4971,7 +4959,7 @@
       <c r="Z31" s="29"/>
       <c r="AA31" s="29"/>
     </row>
-    <row r="32" spans="2:27" s="24" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:27" s="24" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="B32" s="45"/>
       <c r="C32" s="46"/>
       <c r="D32" s="47"/>
@@ -5002,18 +4990,18 @@
       <c r="Z32" s="29"/>
       <c r="AA32" s="29"/>
     </row>
-    <row r="33" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="53"/>
       <c r="C33" s="54"/>
       <c r="D33" s="55"/>
       <c r="E33" s="125">
         <v>1</v>
       </c>
-      <c r="F33" s="174" t="s">
+      <c r="F33" s="216" t="s">
         <v>54</v>
       </c>
-      <c r="G33" s="175"/>
-      <c r="H33" s="176"/>
+      <c r="G33" s="217"/>
+      <c r="H33" s="218"/>
       <c r="I33" s="56"/>
       <c r="J33" s="57"/>
       <c r="K33" s="57"/>
@@ -5033,18 +5021,18 @@
       <c r="Z33" s="29"/>
       <c r="AA33" s="29"/>
     </row>
-    <row r="34" spans="2:27" s="24" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:27" s="24" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="53"/>
       <c r="C34" s="54"/>
       <c r="D34" s="55"/>
       <c r="E34" s="125">
         <v>2</v>
       </c>
-      <c r="F34" s="165" t="s">
+      <c r="F34" s="210" t="s">
         <v>53</v>
       </c>
-      <c r="G34" s="166"/>
-      <c r="H34" s="167"/>
+      <c r="G34" s="211"/>
+      <c r="H34" s="212"/>
       <c r="I34" s="56"/>
       <c r="J34" s="57"/>
       <c r="K34" s="57"/>
@@ -5064,18 +5052,18 @@
       <c r="Z34" s="29"/>
       <c r="AA34" s="29"/>
     </row>
-    <row r="35" spans="2:27" s="24" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:27" s="24" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="25"/>
       <c r="C35" s="30"/>
       <c r="D35" s="31"/>
       <c r="E35" s="115">
         <v>3</v>
       </c>
-      <c r="F35" s="168" t="s">
+      <c r="F35" s="213" t="s">
         <v>55</v>
       </c>
-      <c r="G35" s="169"/>
-      <c r="H35" s="170"/>
+      <c r="G35" s="214"/>
+      <c r="H35" s="215"/>
       <c r="I35" s="58"/>
       <c r="J35" s="59"/>
       <c r="K35" s="59"/>
@@ -5095,16 +5083,16 @@
       <c r="Z35" s="29"/>
       <c r="AA35" s="29"/>
     </row>
-    <row r="36" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="25"/>
       <c r="C36" s="30"/>
       <c r="D36" s="31"/>
       <c r="E36" s="115">
         <v>4</v>
       </c>
-      <c r="F36" s="165"/>
-      <c r="G36" s="166"/>
-      <c r="H36" s="167"/>
+      <c r="F36" s="210"/>
+      <c r="G36" s="211"/>
+      <c r="H36" s="212"/>
       <c r="I36" s="58"/>
       <c r="J36" s="59"/>
       <c r="K36" s="59"/>
@@ -5124,16 +5112,16 @@
       <c r="Z36" s="29"/>
       <c r="AA36" s="29"/>
     </row>
-    <row r="37" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:27" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="25"/>
       <c r="C37" s="30"/>
       <c r="D37" s="31"/>
       <c r="E37" s="115">
         <v>5</v>
       </c>
-      <c r="F37" s="165"/>
-      <c r="G37" s="166"/>
-      <c r="H37" s="167"/>
+      <c r="F37" s="210"/>
+      <c r="G37" s="211"/>
+      <c r="H37" s="212"/>
       <c r="I37" s="58"/>
       <c r="J37" s="59"/>
       <c r="K37" s="59"/>
@@ -5153,7 +5141,7 @@
       <c r="Z37" s="29"/>
       <c r="AA37" s="29"/>
     </row>
-    <row r="38" spans="2:27" s="24" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:27" s="24" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B38" s="61"/>
       <c r="C38" s="62"/>
       <c r="D38" s="63"/>
@@ -5180,7 +5168,7 @@
       <c r="Z38" s="29"/>
       <c r="AA38" s="29"/>
     </row>
-    <row r="39" spans="2:27" s="24" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:27" s="24" customFormat="1" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B39" s="69"/>
       <c r="C39" s="70"/>
       <c r="D39" s="71"/>
@@ -5209,7 +5197,7 @@
       <c r="Z39" s="29"/>
       <c r="AA39" s="29"/>
     </row>
-    <row r="40" spans="2:27" s="24" customFormat="1" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:27" s="24" customFormat="1" ht="5.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="79"/>
       <c r="C40" s="80"/>
       <c r="D40" s="81"/>
@@ -5237,189 +5225,189 @@
       <c r="Z40" s="29"/>
       <c r="AA40" s="29"/>
     </row>
-    <row r="41" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B41" s="206" t="s">
+    <row r="41" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B41" s="178" t="s">
         <v>32</v>
       </c>
-      <c r="C41" s="206" t="s">
+      <c r="C41" s="178" t="s">
         <v>57</v>
       </c>
-      <c r="D41" s="209" t="s">
+      <c r="D41" s="181" t="s">
         <v>56</v>
       </c>
       <c r="F41" s="87"/>
       <c r="G41" s="88"/>
       <c r="H41" s="88"/>
-      <c r="I41" s="211" t="s">
+      <c r="I41" s="183" t="s">
         <v>43</v>
       </c>
-      <c r="J41" s="182" t="s">
+      <c r="J41" s="185" t="s">
         <v>44</v>
       </c>
-      <c r="K41" s="182" t="s">
+      <c r="K41" s="185" t="s">
         <v>45</v>
       </c>
-      <c r="L41" s="182" t="s">
+      <c r="L41" s="185" t="s">
         <v>46</v>
       </c>
-      <c r="M41" s="182" t="s">
+      <c r="M41" s="185" t="s">
         <v>47</v>
       </c>
-      <c r="N41" s="184" t="s">
+      <c r="N41" s="189" t="s">
         <v>48</v>
       </c>
-      <c r="O41" s="184" t="s">
+      <c r="O41" s="189" t="s">
         <v>49</v>
       </c>
-      <c r="P41" s="184" t="s">
+      <c r="P41" s="189" t="s">
         <v>50</v>
       </c>
-      <c r="Q41" s="184" t="s">
+      <c r="Q41" s="189" t="s">
         <v>51</v>
       </c>
-      <c r="R41" s="184"/>
-      <c r="S41" s="215" t="s">
+      <c r="R41" s="189"/>
+      <c r="S41" s="191" t="s">
         <v>52</v>
       </c>
-      <c r="T41" s="179"/>
-      <c r="U41" s="179"/>
-      <c r="V41" s="179"/>
-      <c r="W41" s="187"/>
+      <c r="T41" s="194"/>
+      <c r="U41" s="194"/>
+      <c r="V41" s="194"/>
+      <c r="W41" s="207"/>
       <c r="Y41" s="28"/>
       <c r="Z41" s="29"/>
       <c r="AA41" s="29"/>
     </row>
-    <row r="42" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="207"/>
-      <c r="C42" s="207"/>
-      <c r="D42" s="209"/>
+    <row r="42" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B42" s="179"/>
+      <c r="C42" s="179"/>
+      <c r="D42" s="181"/>
       <c r="F42" s="89"/>
       <c r="G42" s="88"/>
       <c r="H42" s="88"/>
-      <c r="I42" s="211"/>
-      <c r="J42" s="182"/>
-      <c r="K42" s="182"/>
-      <c r="L42" s="182"/>
-      <c r="M42" s="182"/>
-      <c r="N42" s="184"/>
-      <c r="O42" s="184"/>
-      <c r="P42" s="184"/>
-      <c r="Q42" s="184"/>
-      <c r="R42" s="184"/>
-      <c r="S42" s="216"/>
-      <c r="T42" s="180"/>
-      <c r="U42" s="180"/>
-      <c r="V42" s="179"/>
-      <c r="W42" s="188"/>
+      <c r="I42" s="183"/>
+      <c r="J42" s="185"/>
+      <c r="K42" s="185"/>
+      <c r="L42" s="185"/>
+      <c r="M42" s="185"/>
+      <c r="N42" s="189"/>
+      <c r="O42" s="189"/>
+      <c r="P42" s="189"/>
+      <c r="Q42" s="189"/>
+      <c r="R42" s="189"/>
+      <c r="S42" s="192"/>
+      <c r="T42" s="195"/>
+      <c r="U42" s="195"/>
+      <c r="V42" s="194"/>
+      <c r="W42" s="208"/>
       <c r="Y42" s="28"/>
       <c r="Z42" s="29"/>
       <c r="AA42" s="29"/>
     </row>
-    <row r="43" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="207"/>
-      <c r="C43" s="207"/>
-      <c r="D43" s="209"/>
+    <row r="43" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B43" s="179"/>
+      <c r="C43" s="179"/>
+      <c r="D43" s="181"/>
       <c r="F43" s="89"/>
       <c r="G43" s="88"/>
       <c r="H43" s="88"/>
-      <c r="I43" s="211"/>
-      <c r="J43" s="182"/>
-      <c r="K43" s="182"/>
-      <c r="L43" s="182"/>
-      <c r="M43" s="182"/>
-      <c r="N43" s="184"/>
-      <c r="O43" s="184"/>
-      <c r="P43" s="184"/>
-      <c r="Q43" s="184"/>
-      <c r="R43" s="184"/>
-      <c r="S43" s="216"/>
-      <c r="T43" s="180"/>
-      <c r="U43" s="180"/>
-      <c r="V43" s="179"/>
-      <c r="W43" s="188"/>
+      <c r="I43" s="183"/>
+      <c r="J43" s="185"/>
+      <c r="K43" s="185"/>
+      <c r="L43" s="185"/>
+      <c r="M43" s="185"/>
+      <c r="N43" s="189"/>
+      <c r="O43" s="189"/>
+      <c r="P43" s="189"/>
+      <c r="Q43" s="189"/>
+      <c r="R43" s="189"/>
+      <c r="S43" s="192"/>
+      <c r="T43" s="195"/>
+      <c r="U43" s="195"/>
+      <c r="V43" s="194"/>
+      <c r="W43" s="208"/>
       <c r="Y43" s="28"/>
       <c r="Z43" s="29"/>
       <c r="AA43" s="29"/>
     </row>
-    <row r="44" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="207"/>
-      <c r="C44" s="207"/>
-      <c r="D44" s="209"/>
+    <row r="44" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B44" s="179"/>
+      <c r="C44" s="179"/>
+      <c r="D44" s="181"/>
       <c r="F44" s="90"/>
       <c r="G44" s="88"/>
       <c r="H44" s="88"/>
-      <c r="I44" s="211"/>
-      <c r="J44" s="182"/>
-      <c r="K44" s="182"/>
-      <c r="L44" s="182"/>
-      <c r="M44" s="182"/>
-      <c r="N44" s="184"/>
-      <c r="O44" s="184"/>
-      <c r="P44" s="184"/>
-      <c r="Q44" s="184"/>
-      <c r="R44" s="184"/>
-      <c r="S44" s="216"/>
-      <c r="T44" s="180"/>
-      <c r="U44" s="180"/>
-      <c r="V44" s="179"/>
-      <c r="W44" s="188"/>
+      <c r="I44" s="183"/>
+      <c r="J44" s="185"/>
+      <c r="K44" s="185"/>
+      <c r="L44" s="185"/>
+      <c r="M44" s="185"/>
+      <c r="N44" s="189"/>
+      <c r="O44" s="189"/>
+      <c r="P44" s="189"/>
+      <c r="Q44" s="189"/>
+      <c r="R44" s="189"/>
+      <c r="S44" s="192"/>
+      <c r="T44" s="195"/>
+      <c r="U44" s="195"/>
+      <c r="V44" s="194"/>
+      <c r="W44" s="208"/>
       <c r="Z44" s="29"/>
       <c r="AA44" s="29"/>
     </row>
-    <row r="45" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B45" s="207"/>
-      <c r="C45" s="207"/>
-      <c r="D45" s="209"/>
+    <row r="45" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B45" s="179"/>
+      <c r="C45" s="179"/>
+      <c r="D45" s="181"/>
       <c r="F45" s="87"/>
       <c r="G45" s="88"/>
       <c r="H45" s="88"/>
-      <c r="I45" s="211"/>
-      <c r="J45" s="182"/>
-      <c r="K45" s="182"/>
-      <c r="L45" s="182"/>
-      <c r="M45" s="182"/>
-      <c r="N45" s="184"/>
-      <c r="O45" s="184"/>
-      <c r="P45" s="184"/>
-      <c r="Q45" s="184"/>
-      <c r="R45" s="184"/>
-      <c r="S45" s="216"/>
-      <c r="T45" s="180"/>
-      <c r="U45" s="180"/>
-      <c r="V45" s="179"/>
-      <c r="W45" s="188"/>
+      <c r="I45" s="183"/>
+      <c r="J45" s="185"/>
+      <c r="K45" s="185"/>
+      <c r="L45" s="185"/>
+      <c r="M45" s="185"/>
+      <c r="N45" s="189"/>
+      <c r="O45" s="189"/>
+      <c r="P45" s="189"/>
+      <c r="Q45" s="189"/>
+      <c r="R45" s="189"/>
+      <c r="S45" s="192"/>
+      <c r="T45" s="195"/>
+      <c r="U45" s="195"/>
+      <c r="V45" s="194"/>
+      <c r="W45" s="208"/>
       <c r="Z45" s="29"/>
       <c r="AA45" s="29"/>
     </row>
-    <row r="46" spans="2:27" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="207"/>
-      <c r="C46" s="207"/>
-      <c r="D46" s="209"/>
+    <row r="46" spans="2:27" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B46" s="179"/>
+      <c r="C46" s="179"/>
+      <c r="D46" s="181"/>
       <c r="F46" s="91"/>
       <c r="G46" s="88"/>
       <c r="H46" s="88"/>
-      <c r="I46" s="212"/>
-      <c r="J46" s="183"/>
-      <c r="K46" s="183"/>
-      <c r="L46" s="183"/>
-      <c r="M46" s="183"/>
-      <c r="N46" s="185"/>
-      <c r="O46" s="185"/>
-      <c r="P46" s="185"/>
-      <c r="Q46" s="185"/>
-      <c r="R46" s="185"/>
-      <c r="S46" s="217"/>
-      <c r="T46" s="181"/>
-      <c r="U46" s="181"/>
-      <c r="V46" s="186"/>
-      <c r="W46" s="189"/>
+      <c r="I46" s="184"/>
+      <c r="J46" s="186"/>
+      <c r="K46" s="186"/>
+      <c r="L46" s="186"/>
+      <c r="M46" s="186"/>
+      <c r="N46" s="190"/>
+      <c r="O46" s="190"/>
+      <c r="P46" s="190"/>
+      <c r="Q46" s="190"/>
+      <c r="R46" s="190"/>
+      <c r="S46" s="193"/>
+      <c r="T46" s="196"/>
+      <c r="U46" s="196"/>
+      <c r="V46" s="206"/>
+      <c r="W46" s="209"/>
       <c r="Z46" s="2"/>
       <c r="AA46" s="2"/>
     </row>
-    <row r="47" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B47" s="207"/>
-      <c r="C47" s="207"/>
-      <c r="D47" s="209"/>
+    <row r="47" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B47" s="179"/>
+      <c r="C47" s="179"/>
+      <c r="D47" s="181"/>
       <c r="F47" s="91"/>
       <c r="G47" s="91"/>
       <c r="H47" s="91"/>
@@ -5438,15 +5426,15 @@
       <c r="U47" s="93"/>
       <c r="V47" s="93"/>
       <c r="W47" s="94"/>
-      <c r="Z47" s="190" t="s">
+      <c r="Z47" s="203" t="s">
         <v>6</v>
       </c>
-      <c r="AA47" s="190"/>
-    </row>
-    <row r="48" spans="2:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="207"/>
-      <c r="C48" s="207"/>
-      <c r="D48" s="209"/>
+      <c r="AA47" s="203"/>
+    </row>
+    <row r="48" spans="2:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B48" s="179"/>
+      <c r="C48" s="179"/>
+      <c r="D48" s="181"/>
       <c r="E48" s="95"/>
       <c r="F48" s="91"/>
       <c r="G48" s="89"/>
@@ -5476,10 +5464,10 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="207"/>
-      <c r="C49" s="207"/>
-      <c r="D49" s="209"/>
+    <row r="49" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B49" s="179"/>
+      <c r="C49" s="179"/>
+      <c r="D49" s="181"/>
       <c r="F49" s="87"/>
       <c r="G49" s="89"/>
       <c r="H49" s="89"/>
@@ -5504,10 +5492,10 @@
       <c r="Z49" s="144"/>
       <c r="AA49" s="101"/>
     </row>
-    <row r="50" spans="2:27" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B50" s="207"/>
-      <c r="C50" s="207"/>
-      <c r="D50" s="209"/>
+    <row r="50" spans="2:27" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B50" s="179"/>
+      <c r="C50" s="179"/>
+      <c r="D50" s="181"/>
       <c r="F50" s="87"/>
       <c r="G50" s="89"/>
       <c r="H50" s="102"/>
@@ -5532,10 +5520,10 @@
       <c r="Z50" s="144"/>
       <c r="AA50" s="103"/>
     </row>
-    <row r="51" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B51" s="207"/>
-      <c r="C51" s="207"/>
-      <c r="D51" s="209"/>
+    <row r="51" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B51" s="179"/>
+      <c r="C51" s="179"/>
+      <c r="D51" s="181"/>
       <c r="F51" s="87"/>
       <c r="G51" s="87"/>
       <c r="H51" s="87"/>
@@ -5560,10 +5548,10 @@
       <c r="Z51" s="144"/>
       <c r="AA51" s="101"/>
     </row>
-    <row r="52" spans="2:27" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B52" s="207"/>
-      <c r="C52" s="207"/>
-      <c r="D52" s="209"/>
+    <row r="52" spans="2:27" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B52" s="179"/>
+      <c r="C52" s="179"/>
+      <c r="D52" s="181"/>
       <c r="F52" s="104"/>
       <c r="I52" s="96"/>
       <c r="J52" s="97"/>
@@ -5582,10 +5570,10 @@
       <c r="W52" s="98"/>
       <c r="Z52" s="105"/>
     </row>
-    <row r="53" spans="2:27" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="207"/>
-      <c r="C53" s="207"/>
-      <c r="D53" s="209"/>
+    <row r="53" spans="2:27" ht="15.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B53" s="179"/>
+      <c r="C53" s="179"/>
+      <c r="D53" s="181"/>
       <c r="E53" s="106"/>
       <c r="F53" s="106"/>
       <c r="G53" s="106"/>
@@ -5608,103 +5596,103 @@
       <c r="Z53" s="105"/>
       <c r="AA53" s="105"/>
     </row>
-    <row r="54" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B54" s="207"/>
-      <c r="C54" s="207"/>
-      <c r="D54" s="209"/>
-      <c r="E54" s="191"/>
-      <c r="F54" s="191"/>
-      <c r="G54" s="191"/>
-      <c r="H54" s="191"/>
-      <c r="I54" s="191"/>
-      <c r="J54" s="191"/>
-      <c r="K54" s="191"/>
-      <c r="L54" s="191"/>
-      <c r="M54" s="191"/>
-      <c r="N54" s="191"/>
-      <c r="O54" s="191"/>
-      <c r="P54" s="191"/>
-      <c r="Q54" s="191"/>
-      <c r="R54" s="191"/>
-      <c r="S54" s="191"/>
-      <c r="T54" s="191"/>
-      <c r="U54" s="191"/>
-      <c r="V54" s="191"/>
-      <c r="W54" s="192"/>
-    </row>
-    <row r="55" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B55" s="207"/>
-      <c r="C55" s="207"/>
-      <c r="D55" s="209"/>
-      <c r="E55" s="172"/>
-      <c r="F55" s="172"/>
-      <c r="G55" s="172"/>
-      <c r="H55" s="172"/>
-      <c r="I55" s="172"/>
-      <c r="J55" s="172"/>
-      <c r="K55" s="172"/>
-      <c r="L55" s="172"/>
-      <c r="M55" s="172"/>
-      <c r="N55" s="172"/>
-      <c r="O55" s="172"/>
-      <c r="P55" s="172"/>
-      <c r="Q55" s="172"/>
-      <c r="R55" s="172"/>
-      <c r="S55" s="172"/>
-      <c r="T55" s="172"/>
-      <c r="U55" s="172"/>
-      <c r="V55" s="172"/>
-      <c r="W55" s="173"/>
-    </row>
-    <row r="56" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B56" s="207"/>
-      <c r="C56" s="207"/>
-      <c r="D56" s="209"/>
-      <c r="E56" s="172"/>
-      <c r="F56" s="172"/>
-      <c r="G56" s="172"/>
-      <c r="H56" s="172"/>
-      <c r="I56" s="172"/>
-      <c r="J56" s="172"/>
-      <c r="K56" s="172"/>
-      <c r="L56" s="172"/>
-      <c r="M56" s="172"/>
-      <c r="N56" s="172"/>
-      <c r="O56" s="172"/>
-      <c r="P56" s="172"/>
-      <c r="Q56" s="172"/>
-      <c r="R56" s="172"/>
-      <c r="S56" s="172"/>
-      <c r="T56" s="172"/>
-      <c r="U56" s="172"/>
-      <c r="V56" s="172"/>
-      <c r="W56" s="173"/>
-    </row>
-    <row r="57" spans="2:27" ht="64.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="208"/>
-      <c r="C57" s="208"/>
-      <c r="D57" s="210"/>
-      <c r="E57" s="213"/>
-      <c r="F57" s="213"/>
-      <c r="G57" s="213"/>
-      <c r="H57" s="213"/>
-      <c r="I57" s="213"/>
-      <c r="J57" s="213"/>
-      <c r="K57" s="213"/>
-      <c r="L57" s="213"/>
-      <c r="M57" s="213"/>
-      <c r="N57" s="213"/>
-      <c r="O57" s="213"/>
-      <c r="P57" s="213"/>
-      <c r="Q57" s="213"/>
-      <c r="R57" s="213"/>
-      <c r="S57" s="213"/>
-      <c r="T57" s="213"/>
-      <c r="U57" s="213"/>
-      <c r="V57" s="213"/>
-      <c r="W57" s="214"/>
-    </row>
-    <row r="59" spans="2:27" x14ac:dyDescent="0.2">
+    <row r="54" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B54" s="179"/>
+      <c r="C54" s="179"/>
+      <c r="D54" s="181"/>
+      <c r="E54" s="198"/>
+      <c r="F54" s="198"/>
+      <c r="G54" s="198"/>
+      <c r="H54" s="198"/>
+      <c r="I54" s="198"/>
+      <c r="J54" s="198"/>
+      <c r="K54" s="198"/>
+      <c r="L54" s="198"/>
+      <c r="M54" s="198"/>
+      <c r="N54" s="198"/>
+      <c r="O54" s="198"/>
+      <c r="P54" s="198"/>
+      <c r="Q54" s="198"/>
+      <c r="R54" s="198"/>
+      <c r="S54" s="198"/>
+      <c r="T54" s="198"/>
+      <c r="U54" s="198"/>
+      <c r="V54" s="198"/>
+      <c r="W54" s="199"/>
+    </row>
+    <row r="55" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B55" s="179"/>
+      <c r="C55" s="179"/>
+      <c r="D55" s="181"/>
+      <c r="E55" s="201"/>
+      <c r="F55" s="201"/>
+      <c r="G55" s="201"/>
+      <c r="H55" s="201"/>
+      <c r="I55" s="201"/>
+      <c r="J55" s="201"/>
+      <c r="K55" s="201"/>
+      <c r="L55" s="201"/>
+      <c r="M55" s="201"/>
+      <c r="N55" s="201"/>
+      <c r="O55" s="201"/>
+      <c r="P55" s="201"/>
+      <c r="Q55" s="201"/>
+      <c r="R55" s="201"/>
+      <c r="S55" s="201"/>
+      <c r="T55" s="201"/>
+      <c r="U55" s="201"/>
+      <c r="V55" s="201"/>
+      <c r="W55" s="202"/>
+    </row>
+    <row r="56" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B56" s="179"/>
+      <c r="C56" s="179"/>
+      <c r="D56" s="181"/>
+      <c r="E56" s="201"/>
+      <c r="F56" s="201"/>
+      <c r="G56" s="201"/>
+      <c r="H56" s="201"/>
+      <c r="I56" s="201"/>
+      <c r="J56" s="201"/>
+      <c r="K56" s="201"/>
+      <c r="L56" s="201"/>
+      <c r="M56" s="201"/>
+      <c r="N56" s="201"/>
+      <c r="O56" s="201"/>
+      <c r="P56" s="201"/>
+      <c r="Q56" s="201"/>
+      <c r="R56" s="201"/>
+      <c r="S56" s="201"/>
+      <c r="T56" s="201"/>
+      <c r="U56" s="201"/>
+      <c r="V56" s="201"/>
+      <c r="W56" s="202"/>
+    </row>
+    <row r="57" spans="2:27" ht="64.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B57" s="180"/>
+      <c r="C57" s="180"/>
+      <c r="D57" s="182"/>
+      <c r="E57" s="187"/>
+      <c r="F57" s="187"/>
+      <c r="G57" s="187"/>
+      <c r="H57" s="187"/>
+      <c r="I57" s="187"/>
+      <c r="J57" s="187"/>
+      <c r="K57" s="187"/>
+      <c r="L57" s="187"/>
+      <c r="M57" s="187"/>
+      <c r="N57" s="187"/>
+      <c r="O57" s="187"/>
+      <c r="P57" s="187"/>
+      <c r="Q57" s="187"/>
+      <c r="R57" s="187"/>
+      <c r="S57" s="187"/>
+      <c r="T57" s="187"/>
+      <c r="U57" s="187"/>
+      <c r="V57" s="187"/>
+      <c r="W57" s="188"/>
+    </row>
+    <row r="59" spans="2:27" ht="13" x14ac:dyDescent="0.3">
       <c r="K59" s="110" t="s">
         <v>11</v>
       </c>
@@ -5724,10 +5712,10 @@
       <c r="S59" s="119" t="s">
         <v>15</v>
       </c>
-      <c r="T59" s="177" t="s">
+      <c r="T59" s="204" t="s">
         <v>21</v>
       </c>
-      <c r="U59" s="178"/>
+      <c r="U59" s="205"/>
       <c r="V59" s="111"/>
       <c r="W59" s="111"/>
       <c r="X59" s="111"/>
@@ -5735,7 +5723,7 @@
       <c r="Z59" s="111"/>
       <c r="AA59" s="111"/>
     </row>
-    <row r="60" spans="2:27" x14ac:dyDescent="0.2">
+    <row r="60" spans="2:27" ht="13" x14ac:dyDescent="0.3">
       <c r="J60" s="3" t="s">
         <v>14</v>
       </c>
@@ -5758,10 +5746,10 @@
       <c r="S60" s="132" t="s">
         <v>16</v>
       </c>
-      <c r="T60" s="177" t="s">
+      <c r="T60" s="204" t="s">
         <v>22</v>
       </c>
-      <c r="U60" s="178"/>
+      <c r="U60" s="205"/>
       <c r="V60" s="113"/>
       <c r="W60" s="113"/>
       <c r="X60" s="113"/>
@@ -5769,36 +5757,36 @@
       <c r="Z60" s="113"/>
       <c r="AA60" s="113"/>
     </row>
-    <row r="61" spans="2:27" x14ac:dyDescent="0.2">
+    <row r="61" spans="2:27" ht="13" x14ac:dyDescent="0.3">
       <c r="S61" s="142" t="s">
         <v>17</v>
       </c>
-      <c r="T61" s="177" t="s">
+      <c r="T61" s="204" t="s">
         <v>23</v>
       </c>
-      <c r="U61" s="178"/>
+      <c r="U61" s="205"/>
       <c r="Y61" s="1"/>
       <c r="Z61" s="1"/>
       <c r="AA61" s="1"/>
     </row>
-    <row r="62" spans="2:27" x14ac:dyDescent="0.2">
+    <row r="62" spans="2:27" x14ac:dyDescent="0.25">
       <c r="Y62" s="1"/>
       <c r="Z62" s="1"/>
       <c r="AA62" s="1"/>
     </row>
-    <row r="63" spans="2:27" x14ac:dyDescent="0.2">
+    <row r="63" spans="2:27" x14ac:dyDescent="0.25">
       <c r="K63" s="147"/>
       <c r="L63" s="150" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="64" spans="2:27" x14ac:dyDescent="0.2">
+    <row r="64" spans="2:27" x14ac:dyDescent="0.25">
       <c r="K64" s="148"/>
       <c r="L64" s="150" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="65" spans="11:12" x14ac:dyDescent="0.2">
+    <row r="65" spans="11:12" x14ac:dyDescent="0.25">
       <c r="K65" s="149"/>
       <c r="L65" s="150" t="s">
         <v>27</v>
@@ -5806,6 +5794,50 @@
     </row>
   </sheetData>
   <mergeCells count="60">
+    <mergeCell ref="F34:H34"/>
+    <mergeCell ref="F36:H36"/>
+    <mergeCell ref="F37:H37"/>
+    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="F28:H28"/>
+    <mergeCell ref="F29:H29"/>
+    <mergeCell ref="F30:H30"/>
+    <mergeCell ref="F33:H33"/>
+    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="F24:H24"/>
+    <mergeCell ref="F25:H25"/>
+    <mergeCell ref="F26:H26"/>
+    <mergeCell ref="F27:H27"/>
+    <mergeCell ref="F18:H18"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="F21:H21"/>
+    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="F13:H13"/>
+    <mergeCell ref="F14:H14"/>
+    <mergeCell ref="F15:H15"/>
+    <mergeCell ref="F16:H16"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="F9:H9"/>
+    <mergeCell ref="F10:H10"/>
+    <mergeCell ref="F11:H11"/>
+    <mergeCell ref="F12:H12"/>
+    <mergeCell ref="T61:U61"/>
+    <mergeCell ref="E56:W56"/>
+    <mergeCell ref="U41:U46"/>
+    <mergeCell ref="L41:L46"/>
+    <mergeCell ref="M41:M46"/>
+    <mergeCell ref="N41:N46"/>
+    <mergeCell ref="O41:O46"/>
+    <mergeCell ref="P41:P46"/>
+    <mergeCell ref="Q41:Q46"/>
+    <mergeCell ref="V41:V46"/>
+    <mergeCell ref="W41:W46"/>
+    <mergeCell ref="Z47:AA47"/>
+    <mergeCell ref="E54:W54"/>
+    <mergeCell ref="E55:W55"/>
+    <mergeCell ref="T59:U59"/>
+    <mergeCell ref="T60:U60"/>
     <mergeCell ref="E3:W4"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="I5:R5"/>
@@ -5822,50 +5854,6 @@
     <mergeCell ref="T41:T46"/>
     <mergeCell ref="F6:H6"/>
     <mergeCell ref="F7:H7"/>
-    <mergeCell ref="Z47:AA47"/>
-    <mergeCell ref="E54:W54"/>
-    <mergeCell ref="E55:W55"/>
-    <mergeCell ref="T59:U59"/>
-    <mergeCell ref="T60:U60"/>
-    <mergeCell ref="T61:U61"/>
-    <mergeCell ref="E56:W56"/>
-    <mergeCell ref="U41:U46"/>
-    <mergeCell ref="L41:L46"/>
-    <mergeCell ref="M41:M46"/>
-    <mergeCell ref="N41:N46"/>
-    <mergeCell ref="O41:O46"/>
-    <mergeCell ref="P41:P46"/>
-    <mergeCell ref="Q41:Q46"/>
-    <mergeCell ref="V41:V46"/>
-    <mergeCell ref="W41:W46"/>
-    <mergeCell ref="F8:H8"/>
-    <mergeCell ref="F9:H9"/>
-    <mergeCell ref="F10:H10"/>
-    <mergeCell ref="F11:H11"/>
-    <mergeCell ref="F12:H12"/>
-    <mergeCell ref="F13:H13"/>
-    <mergeCell ref="F14:H14"/>
-    <mergeCell ref="F15:H15"/>
-    <mergeCell ref="F16:H16"/>
-    <mergeCell ref="F17:H17"/>
-    <mergeCell ref="F18:H18"/>
-    <mergeCell ref="F19:H19"/>
-    <mergeCell ref="F20:H20"/>
-    <mergeCell ref="F21:H21"/>
-    <mergeCell ref="F22:H22"/>
-    <mergeCell ref="F23:H23"/>
-    <mergeCell ref="F24:H24"/>
-    <mergeCell ref="F25:H25"/>
-    <mergeCell ref="F26:H26"/>
-    <mergeCell ref="F27:H27"/>
-    <mergeCell ref="F34:H34"/>
-    <mergeCell ref="F36:H36"/>
-    <mergeCell ref="F37:H37"/>
-    <mergeCell ref="F35:H35"/>
-    <mergeCell ref="F28:H28"/>
-    <mergeCell ref="F29:H29"/>
-    <mergeCell ref="F30:H30"/>
-    <mergeCell ref="F33:H33"/>
   </mergeCells>
   <conditionalFormatting sqref="B40:D40">
     <cfRule type="cellIs" dxfId="22" priority="58" stopIfTrue="1" operator="notEqual">

</xml_diff>